<commit_message>
Nilo: proximo check-in 21/11 + foco ajustado para peitoral e perda de gordura
</commit_message>
<xml_diff>
--- a/gerador/modelo-treinos.xlsx
+++ b/gerador/modelo-treinos.xlsx
@@ -805,22 +805,22 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Foco: perda de gordura e hipertrofia · Musculação 4x (Peito/Costas/Pernas/Ombro+Braço) + atividade livre 3x</t>
+          <t>Foco: perda de gordura e hipertrofia de peitorais · Musculação 4x (Peito/Costas/Pernas/Ombro+Braço) + atividade livre 3x</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>PERDA DE GORDURA E HIPERTROFIA</t>
+          <t>PERDA DE GORDURA E HIPERTROFIA DE PEITORAL</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Novo ciclo com split clássico: segunda peito, terça costas, quarta pernas, quinta ombros/bíceps/tríceps. A musculação (4x) fecha o déficit calórico junto com os 3 dias de atividade livre, por conta do próprio Nilo (CrossFit, cardio ou o que preferir nos dias livres).</t>
+          <t>Ciclo com prioridade em peitoral: split clássico (segunda peito, terça costas, quarta pernas, quinta ombros/bíceps/tríceps), com o treino de peito estruturado para máximo estímulo (bi-set e drop set). A musculação (4x) fecha o déficit calórico junto com os 3 dias de atividade livre, por conta do próprio Nilo (CrossFit, cardio ou o que preferir nos dias livres).</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>01/07/2026</t>
+          <t>21/11/2026</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -2563,10 +2563,6 @@
           <t>Em breve</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr"/>
-      <c r="F38" t="inlineStr"/>
-      <c r="G38" t="inlineStr"/>
-      <c r="H38" t="inlineStr"/>
       <c r="I38" t="inlineStr">
         <is>
           <t>Treino sendo finalizado, chega em breve.</t>
@@ -2594,10 +2590,6 @@
           <t>Em breve</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr"/>
-      <c r="F39" t="inlineStr"/>
-      <c r="G39" t="inlineStr"/>
-      <c r="H39" t="inlineStr"/>
       <c r="I39" t="inlineStr">
         <is>
           <t>Treino sendo finalizado, chega em breve.</t>
@@ -2625,10 +2617,6 @@
           <t>Em breve</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr"/>
-      <c r="F40" t="inlineStr"/>
-      <c r="G40" t="inlineStr"/>
-      <c r="H40" t="inlineStr"/>
       <c r="I40" t="inlineStr">
         <is>
           <t>Treino sendo finalizado, chega em breve.</t>

</xml_diff>

<commit_message>
Adiciona aluna Marina Barbato (musculacao 5x - foco gluteos e ombros)
</commit_message>
<xml_diff>
--- a/gerador/modelo-treinos.xlsx
+++ b/gerador/modelo-treinos.xlsx
@@ -536,7 +536,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N7"/>
+  <dimension ref="A1:N8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -972,6 +972,61 @@
         <v>1</v>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Marina Barbato</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>A definir</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Foco: perda de gordura com ênfase em glúteos e ombros · Musculação 5x (Quadríceps/Dorsal/Posterior de coxa/Ombro+Tríceps+Bíceps/Glúteos) + bike aeróbica seg-sáb</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>PERDA DE GORDURA COM ÊNFASE EM GLÚTEOS E OMBROS</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Foco em emagrecimento com ênfase em glúteos e ombros. Musculação 5x por semana (quadríceps, dorsal, posterior de coxa, ombro/tríceps/bíceps e glúteos) combinada com bike aeróbica de segunda a sábado, domingo de descanso. Progressão de carga e técnica correta em cada sessão.</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>A definir</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>5x musculação + bike (seg-sáb)</t>
+        </is>
+      </c>
+      <c r="N8" t="n">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -983,7 +1038,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J107"/>
+  <dimension ref="A1:J133"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -5331,6 +5386,1050 @@
           <t>Corpo alinhado da cabeça ao calcanhar, abdômen contraído.</t>
         </is>
       </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>Marina Barbato</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>A · Seg · Quadríceps</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>Agachamento livre (ativação)</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>Quadríceps</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr"/>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>Descida lenta (excêntrica controlada) — séries de ativação antes da carga.</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>Marina Barbato</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>A · Seg · Quadríceps</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>Agachamento livre (carga)</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>Quadríceps</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr"/>
+      <c r="I109" t="inlineStr">
+        <is>
+          <t>Séries de trabalho, na sequência das 2 séries de ativação.</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>Marina Barbato</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>A · Seg · Quadríceps</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>Leg press 45°</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>Quadríceps</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>20/15/12/10/8</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr"/>
+      <c r="I110" t="inlineStr">
+        <is>
+          <t>Progressão de carga a cada série.</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>Marina Barbato</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>A · Seg · Quadríceps</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>Cadeira extensora</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>Quadríceps</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr"/>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>Marina Barbato</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>A · Seg · Quadríceps</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>Cadeira extensora</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>Quadríceps</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr"/>
+      <c r="I112" t="inlineStr">
+        <is>
+          <t>Segundo bloco — aumentar a carga.</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>Marina Barbato</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>A · Seg · Quadríceps</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>Panturrilha em pé</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>Panturrilha</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="H113" t="inlineStr"/>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>Marina Barbato</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>B · Ter · Dorsal</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>Remada sentada pulley</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>Dorsal</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr"/>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>Bi-set com a rosca direta com halteres (próximo exercício), sem descanso entre eles.</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>Marina Barbato</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>B · Ter · Dorsal</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>Rosca direta halteres</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>Bíceps</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="H115" t="inlineStr"/>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>Bi-set com a remada sentada pulley (exercício anterior).</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>Marina Barbato</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>B · Ter · Dorsal</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>Puxador aberto pulley</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>Dorsal</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>15/12/10/8</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr"/>
+      <c r="I116" t="inlineStr">
+        <is>
+          <t>Progressão de carga a cada série.</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>Marina Barbato</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>B · Ter · Dorsal</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>Remo aeróbico</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>Cardio</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr"/>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>10 min</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr"/>
+      <c r="I117" t="inlineStr">
+        <is>
+          <t>Ritmo moderado-intenso.</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>Marina Barbato</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>B · Ter · Dorsal</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>Banco romano</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>Lombar/Posterior</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="H118" t="inlineStr"/>
+      <c r="I118" t="inlineStr">
+        <is>
+          <t>Descida lenta (excêntrica controlada).</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>Marina Barbato</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>C · Qua · Posterior de coxa</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>Mesa flexora</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>Posterior de coxa</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="H119" t="inlineStr"/>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>Marina Barbato</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>C · Qua · Posterior de coxa</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>Mesa flexora</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>Posterior de coxa</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="H120" t="inlineStr"/>
+      <c r="I120" t="inlineStr">
+        <is>
+          <t>Segundo bloco — aumentar a carga.</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>Marina Barbato</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>C · Qua · Posterior de coxa</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>Flexor de joelhos em pé</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>Posterior de coxa</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="H121" t="inlineStr"/>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>Marina Barbato</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>C · Qua · Posterior de coxa</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>Stiff halteres</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>Posterior de coxa/Glúteo</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr"/>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>Marina Barbato</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>C · Qua · Posterior de coxa</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>Abdominal máquina</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>Abdômen</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="H123" t="inlineStr"/>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>Marina Barbato</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>D · Qui · Ombro, Tríceps e Bíceps</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>Manguito rotador (elástico ou pulley)</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>Ombro</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="H124" t="inlineStr"/>
+      <c r="I124" t="inlineStr">
+        <is>
+          <t>Ativação do manguito rotador antes da carga.</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>Marina Barbato</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>D · Qui · Ombro, Tríceps e Bíceps</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>Elevação lateral halteres</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>Ombro</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="H125" t="inlineStr"/>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>Marina Barbato</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>D · Qui · Ombro, Tríceps e Bíceps</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>Elevação lateral no pulley</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>Ombro</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="H126" t="inlineStr"/>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>Marina Barbato</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>D · Qui · Ombro, Tríceps e Bíceps</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>Desenvolvimento fechado halteres</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>Ombro</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="H127" t="inlineStr"/>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>Marina Barbato</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>D · Qui · Ombro, Tríceps e Bíceps</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>Tríceps pulley corda</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>Tríceps</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="H128" t="inlineStr"/>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>Marina Barbato</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>E · Sex · Glúteos</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>Supino sentada</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>Glúteo</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="H129" t="inlineStr"/>
+      <c r="I129" t="inlineStr">
+        <is>
+          <t>Confirmar nome do aparelho com a Larissa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>Marina Barbato</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>E · Sex · Glúteos</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>Cadeira abdutora</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>Glúteo médio</t>
+        </is>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="H130" t="inlineStr"/>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>Marina Barbato</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>E · Sex · Glúteos</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>Elevação pélvica</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>Glúteo</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="H131" t="inlineStr"/>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>Marina Barbato</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>E · Sex · Glúteos</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>Glúteo no pulley (extensão de quadril)</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>Glúteo</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="H132" t="inlineStr"/>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>Marina Barbato</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>E · Sex · Glúteos</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>Glúteo — chute na máquina</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>Glúteo</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G133" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="H133" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Nilo: completa ciclo - costas (ter), pernas presencial (qua), ombros (qui), biceps/triceps (sex)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/gerador/modelo-treinos.xlsx
+++ b/gerador/modelo-treinos.xlsx
@@ -805,7 +805,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Foco: perda de gordura e hipertrofia de peitorais · Musculação 4x (Peito/Costas/Pernas/Ombro+Braço) + atividade livre 3x</t>
+          <t>Foco: perda de gordura e hipertrofia de peitorais · Musculação 5x (Peito/Costas/Pernas presencial/Ombros/Bíceps+Tríceps) + atividade livre</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -815,7 +815,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Ciclo com prioridade em peitoral: split clássico (segunda peito, terça costas, quarta pernas, quinta ombros/bíceps/tríceps), com o treino de peito estruturado para máximo estímulo (bi-set e drop set). A musculação (4x) fecha o déficit calórico junto com os 3 dias de atividade livre, por conta do próprio Nilo (CrossFit, cardio ou o que preferir nos dias livres).</t>
+          <t>Ciclo com prioridade em peitoral: segunda peito, terça costas, quarta pernas (presencial comigo), quinta ombros e sexta bíceps/tríceps, com o treino de peito estruturado para máximo estímulo (bi-set e drop set). A musculação fecha o déficit calórico junto com a atividade livre, por conta do próprio Nilo (CrossFit, cardio ou o que preferir nos dias livres).</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -845,7 +845,7 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>4x musculação + 3x atividade livre</t>
+          <t>5x musculação + atividade livre</t>
         </is>
       </c>
       <c r="N5" t="n">
@@ -1038,7 +1038,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J133"/>
+  <dimension ref="A1:J146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2615,12 +2615,27 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Em breve</t>
+          <t>Graviton (barra)</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Costas</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>15</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>Treino sendo finalizado, chega em breve.</t>
+          <t>Controla a descida, peito aberto e escápulas encaixadas.</t>
         </is>
       </c>
     </row>
@@ -2632,22 +2647,37 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>C · Qua · Pernas</t>
+          <t>B · Ter · Costas</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Em breve</t>
+          <t>Puxador aberto articulado</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Costas</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>12/12/12/12</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>Treino sendo finalizado, chega em breve.</t>
+          <t>Progressão de carga: mantém as 12 reps e aumenta a carga a cada série.</t>
         </is>
       </c>
     </row>
@@ -2659,49 +2689,64 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>D · Qui · Ombros, Bíceps e Tríceps</t>
+          <t>B · Ter · Costas</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Em breve</t>
+          <t>Remada sentada na máquina</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Costas</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>15</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>Treino sendo finalizado, chega em breve.</t>
+          <t>Segura 2 seg na contração (isometria) em cada rep.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Felipe</t>
+          <t>Nilo Sheeny</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>A · Ter · Peito</t>
+          <t>B · Ter · Costas</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Supino na máquina (chest press)</t>
+          <t>Remada alta no pulley com corda</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Peitoral · principal</t>
+          <t>Deltoide / Trapézio</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -2711,39 +2756,39 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>12/10/8/8</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>Progressão de carga ao longo das séries. Empurra controlado, sem travar o cotovelo no fim.</t>
+          <t>Puxa a corda até a altura do peito com os cotovelos acima das mãos.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Felipe</t>
+          <t>Nilo Sheeny</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>A · Ter · Peito</t>
+          <t>B · Ter · Costas</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Supino inclinado com halteres</t>
+          <t>Encolhimento de ombros no Smith</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Peitoral</t>
+          <t>Trapézio</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -2753,165 +2798,155 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>20</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>Progressão de carga: aumente o peso a cada série mantendo a técnica.</t>
+          <t>Sobe os ombros em direção às orelhas, sem girar; segura 1 seg no topo.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Felipe</t>
+          <t>Nilo Sheeny</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>A · Ter · Peito</t>
+          <t>C · Qua · Pernas (presencial)</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Crucifixo na máquina (voador)</t>
+          <t>Treino presencial com a Larissa</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Peitoral</t>
-        </is>
-      </c>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="G43" t="inlineStr">
-        <is>
-          <t>12</t>
+          <t>Pernas</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>Abre bem e segura 1 seg na contração.</t>
+          <t>Treino de pernas feito presencialmente comigo. Os exercícios e cargas são passados na hora.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Felipe</t>
+          <t>Nilo Sheeny</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>A · Ter · Peito</t>
+          <t>D · Qui · Ombros</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Crossover na polia</t>
+          <t>Manguito rotador no pulley (rotação externa)</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Peitoral</t>
+          <t>Manguito rotador</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>15/12/10</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>Drop set: tudo na MESMA série, reduz a carga sem descanso (15 → 12 → 10) até a falha.</t>
+          <t>Cotovelo colado ao corpo, gira o antebraço pra fora. Carga leve, movimento controlado.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Felipe</t>
+          <t>Nilo Sheeny</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>A · Ter · Peito</t>
+          <t>D · Qui · Ombros</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Tríceps na corda</t>
+          <t>Desenvolvimento na máquina</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Tríceps</t>
+          <t>Deltoide</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>12/12/12/12</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>Cotovelos fixos junto ao corpo, abre bem no fim.</t>
+          <t>Progressão de carga: mantém as 12 reps e aumenta a carga a cada série.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Felipe</t>
+          <t>Nilo Sheeny</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>A · Ter · Peito</t>
+          <t>D · Qui · Ombros</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Tríceps testa</t>
+          <t>Elevação lateral sentado no banco</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Tríceps</t>
+          <t>Deltoide lateral</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -2933,27 +2968,27 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Felipe</t>
+          <t>Nilo Sheeny</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>B · Qui · Costas</t>
+          <t>D · Qui · Ombros</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Barra fixa ou puxada alta (pegada aberta)</t>
+          <t>Elevação frontal unilateral no pulley</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Costas · principal</t>
+          <t>Deltoide anterior</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -2963,39 +2998,39 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>12/10/8/8</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>Progressão de carga ao longo das séries.</t>
+          <t>Um braço de cada vez, sobe até a altura do ombro e controla a descida.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Felipe</t>
+          <t>Nilo Sheeny</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>B · Qui · Costas</t>
+          <t>D · Qui · Ombros</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Remada sentada na máquina (pegada neutra)</t>
+          <t>Abdominal na máquina</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Costas</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -3005,165 +3040,165 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>12/10/10/08</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>Progressão de carga. Controla a fase negativa.</t>
+          <t>Contrai o abdômen, sem puxar com os braços.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Felipe</t>
+          <t>Nilo Sheeny</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>B · Qui · Costas</t>
+          <t>E · Sex · Bíceps e Tríceps</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Remada cavalinho (T-bar)</t>
+          <t>Rosca direta na máquina</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Costas</t>
+          <t>Bíceps</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>10-12</t>
+          <t>12/12/12/12</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>Peito apoiado, puxa com os cotovelos.</t>
+          <t>Progressão de carga: mantém as 12 reps e aumenta a carga a cada série.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Felipe</t>
+          <t>Nilo Sheeny</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>B · Qui · Costas</t>
+          <t>E · Sex · Bíceps e Tríceps</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Puxada com triângulo (pegada neutra)</t>
+          <t>Tríceps inverso no pulley (barra reta)</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Costas</t>
+          <t>Tríceps</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>15/12/12/12</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>Leva o triângulo ao peito, escápulas pra baixo.</t>
+          <t>Pegada inversa (palmas pra cima). Progressão de carga ao longo das séries.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Felipe</t>
+          <t>Nilo Sheeny</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>B · Qui · Costas</t>
+          <t>E · Sex · Bíceps e Tríceps</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Pullover na polia</t>
+          <t>Rosca scott na máquina</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Costas</t>
+          <t>Bíceps</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>15/12/10</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>Sente o dorsal alongar e contrair, cotovelos semi-fixos.</t>
+          <t>Drop set: tudo na MESMA série, reduz a carga sem descanso (15 → 12 → 10) até a falha.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Felipe</t>
+          <t>Nilo Sheeny</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>B · Qui · Costas</t>
+          <t>E · Sex · Bíceps e Tríceps</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Remada unilateral com halter (serrote)</t>
+          <t>Tríceps no pulley com corda</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Costas</t>
+          <t>Tríceps</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -3173,54 +3208,54 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>10 cada</t>
+          <t>15/12/10</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>Um lado de cada vez, sem rodar o tronco.</t>
+          <t>Drop set: tudo na MESMA série, reduz a carga sem descanso (15 → 12 → 10) até a falha.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Felipe</t>
+          <t>Nilo Sheeny</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>B · Qui · Costas</t>
+          <t>E · Sex · Bíceps e Tríceps</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Rosca scott (banco)</t>
+          <t>Abdominal na máquina</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Bíceps</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>10-12</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>Progressão de carga: aumente o peso a cada série. Cotovelos apoiados no banco, sobe e desce controlado.</t>
+          <t>Contrai o abdômen, sem puxar com os braços.</t>
         </is>
       </c>
     </row>
@@ -3232,22 +3267,22 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>C · Sex · Pernas</t>
+          <t>A · Ter · Peito</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Leg press 45°</t>
+          <t>Supino na máquina (chest press)</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Pernas · principal</t>
+          <t>Peitoral · principal</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -3257,12 +3292,12 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>12/10/10/08</t>
+          <t>12/10/8/8</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>Progressão de carga. Pés na largura do quadril, desce controlado.</t>
+          <t>Progressão de carga ao longo das séries. Empurra controlado, sem travar o cotovelo no fim.</t>
         </is>
       </c>
     </row>
@@ -3274,37 +3309,37 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>C · Sex · Pernas</t>
+          <t>A · Ter · Peito</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Agachamento hack</t>
+          <t>Supino inclinado com halteres</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Quadríceps</t>
+          <t>Peitoral</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>10-12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>Máquina, poupando a coluna que o CrossFit já castiga.</t>
+          <t>Progressão de carga: aumente o peso a cada série mantendo a técnica.</t>
         </is>
       </c>
     </row>
@@ -3316,22 +3351,22 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>C · Sex · Pernas</t>
+          <t>A · Ter · Peito</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Cadeira extensora</t>
+          <t>Crucifixo na máquina (voador)</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Quadríceps</t>
+          <t>Peitoral</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -3341,12 +3376,12 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>15/12/10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>Drop set: tudo na MESMA série, reduz a carga sem descanso (15 → 12 → 10) até a falha.</t>
+          <t>Abre bem e segura 1 seg na contração.</t>
         </is>
       </c>
     </row>
@@ -3358,37 +3393,37 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>C · Sex · Pernas</t>
+          <t>A · Ter · Peito</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Mesa flexora (posterior)</t>
+          <t>Crossover na polia</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Posterior</t>
+          <t>Peitoral</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>12/10/10/10</t>
+          <t>15/12/10</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>Progressão de carga. Controla a fase negativa.</t>
+          <t>Drop set: tudo na MESMA série, reduz a carga sem descanso (15 → 12 → 10) até a falha.</t>
         </is>
       </c>
     </row>
@@ -3400,22 +3435,22 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>C · Sex · Pernas</t>
+          <t>A · Ter · Peito</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Coice de glúteo na polia</t>
+          <t>Tríceps na corda</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Glúteos</t>
+          <t>Tríceps</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -3425,12 +3460,12 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>12 cada</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>Um lado de cada vez, segura 1 seg na contração do glúteo.</t>
+          <t>Cotovelos fixos junto ao corpo, abre bem no fim.</t>
         </is>
       </c>
     </row>
@@ -3442,22 +3477,22 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>C · Sex · Pernas</t>
+          <t>A · Ter · Peito</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Elevação pélvica (glúteo)</t>
+          <t>Tríceps testa</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Glúteos</t>
+          <t>Tríceps</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
@@ -3467,12 +3502,12 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>15/12/10</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>Segura 2 seg no topo (isometria) apertando o glúteo.</t>
+          <t>Drop set: tudo na MESMA série, reduz a carga sem descanso (15 → 12 → 10) até a falha.</t>
         </is>
       </c>
     </row>
@@ -3484,22 +3519,22 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>C · Sex · Pernas</t>
+          <t>B · Qui · Costas</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Panturrilha em pé</t>
+          <t>Barra fixa ou puxada alta (pegada aberta)</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Panturrilha</t>
+          <t>Costas · principal</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
@@ -3509,12 +3544,12 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>20/15/12/12</t>
+          <t>12/10/8/8</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>Drop set na última série + isometria de 2 seg no topo de cada rep.</t>
+          <t>Progressão de carga ao longo das séries.</t>
         </is>
       </c>
     </row>
@@ -3526,32 +3561,37 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>D · Sáb · Corrida</t>
+          <t>B · Qui · Costas</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Aquecimento</t>
+          <t>Remada sentada na máquina (pegada neutra)</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Corrida · aquecimento</t>
+          <t>Costas</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>4</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>5 min</t>
+          <t>12/10/10/08</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>Faça o aquecimento, depois SÓ o bloco da semana atual do seu ciclo, e termine no desaquecimento. A cada 4 semanas o ciclo recomeça, subindo cerca de 10%. Comece com caminhada rápida evoluindo para trote leve.</t>
+          <t>Progressão de carga. Controla a fase negativa.</t>
         </is>
       </c>
     </row>
@@ -3563,32 +3603,37 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>D · Sáb · Corrida</t>
+          <t>B · Qui · Costas</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Semana 1 · Corrida contínua leve</t>
+          <t>Remada cavalinho (T-bar)</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Corrida · Semana 1</t>
+          <t>Costas</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>3</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>4-5 km</t>
+          <t>10-12</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>Ritmo de conversa (Z2): você consegue falar frases inteiras. Registre seu tempo total no fim.</t>
+          <t>Peito apoiado, puxa com os cotovelos.</t>
         </is>
       </c>
     </row>
@@ -3600,37 +3645,37 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>D · Sáb · Corrida</t>
+          <t>B · Qui · Costas</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Semana 2 · Fartlek</t>
+          <t>Puxada com triângulo (pegada neutra)</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Corrida · Semana 2</t>
+          <t>Costas</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>(3 min corrida + 1 min caminhada)</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>6 blocos de 3 min correndo moderado + 1 min caminhando. Registre o tempo total.</t>
+          <t>Leva o triângulo ao peito, escápulas pra baixo.</t>
         </is>
       </c>
     </row>
@@ -3642,32 +3687,37 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>D · Sáb · Corrida</t>
+          <t>B · Qui · Costas</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Semana 3 · Longão leve</t>
+          <t>Pullover na polia</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Corrida · Semana 3</t>
+          <t>Costas</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>3</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>5-6 km</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>Contínuo em Z2, sem pressa, construindo resistência. Registre seu tempo.</t>
+          <t>Sente o dorsal alongar e contrair, cotovelos semi-fixos.</t>
         </is>
       </c>
     </row>
@@ -3679,32 +3729,37 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>D · Sáb · Corrida</t>
+          <t>B · Qui · Costas</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Semana 4 · Progressiva</t>
+          <t>Remada unilateral com halter (serrote)</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Corrida · Semana 4</t>
+          <t>Costas</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>3</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>5 km</t>
+          <t>10 cada</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>Comece leve e termine o último km mais forte (limiar leve). Registre seu tempo.</t>
+          <t>Um lado de cada vez, sem rodar o tronco.</t>
         </is>
       </c>
     </row>
@@ -3716,96 +3771,106 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>D · Sáb · Corrida</t>
+          <t>B · Qui · Costas</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Desaquecimento</t>
+          <t>Rosca scott (banco)</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Corrida · volta à calma</t>
+          <t>Bíceps</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>3</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>5 min</t>
+          <t>10-12</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>Trote bem leve até virar caminhada, depois alongue panturrilha, posterior e quadril.</t>
+          <t>Progressão de carga: aumente o peso a cada série. Cotovelos apoiados no banco, sobe e desce controlado.</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Jaqueline Galo</t>
+          <t>Felipe</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>A · Quadríceps</t>
+          <t>C · Sex · Pernas</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Agachamento cálice</t>
+          <t>Leg press 45°</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Quadríceps</t>
+          <t>Pernas · principal</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>12/10/10/08</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>Progressão de carga. Pés na largura do quadril, desce controlado.</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Jaqueline Galo</t>
+          <t>Felipe</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>A · Quadríceps</t>
+          <t>C · Sex · Pernas</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Afundo alternado no step</t>
+          <t>Agachamento hack</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Pernas/glúteos</t>
+          <t>Quadríceps</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
@@ -3815,24 +3880,29 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>10-12</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>Máquina, poupando a coluna que o CrossFit já castiga.</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Jaqueline Galo</t>
+          <t>Felipe</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>A · Quadríceps</t>
+          <t>C · Sex · Pernas</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -3847,412 +3917,412 @@
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>15/12/10/08</t>
+          <t>15/12/10</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>Progressão de carga ao longo das séries.</t>
+          <t>Drop set: tudo na MESMA série, reduz a carga sem descanso (15 → 12 → 10) até a falha.</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Jaqueline Galo</t>
+          <t>Felipe</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>A · Quadríceps</t>
+          <t>C · Sex · Pernas</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Leg press 45°</t>
+          <t>Mesa flexora (posterior)</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Pernas</t>
+          <t>Posterior</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>12/10/10/10</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>Descida lenta (controlada).</t>
+          <t>Progressão de carga. Controla a fase negativa.</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Jaqueline Galo</t>
+          <t>Felipe</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>A · Quadríceps</t>
+          <t>C · Sex · Pernas</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Escada</t>
+          <t>Coice de glúteo na polia</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Cardio</t>
+          <t>Glúteos</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>3</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>15 min</t>
+          <t>12 cada</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>Um lado de cada vez, segura 1 seg na contração do glúteo.</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Jaqueline Galo</t>
+          <t>Felipe</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>B · Superiores</t>
+          <t>C · Sex · Pernas</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Puxador costas no graviton + Desenvolvimento halteres fechado</t>
+          <t>Elevação pélvica (glúteo)</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Costas/Ombro</t>
+          <t>Glúteos</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>máximo / 10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>Bi-set: sem descanso entre os dois — puxador no graviton até o máximo, seguido de desenvolvimento com halteres fechado (10 reps).</t>
+          <t>Segura 2 seg no topo (isometria) apertando o glúteo.</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Jaqueline Galo</t>
+          <t>Felipe</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>B · Superiores</t>
+          <t>C · Sex · Pernas</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Pulldown barra reta (pulley) + Tríceps pulley</t>
+          <t>Panturrilha em pé</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Costas/Tríceps</t>
+          <t>Panturrilha</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>20/15/12/12</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>Bi-set: sem descanso entre os dois.</t>
+          <t>Drop set na última série + isometria de 2 seg no topo de cada rep.</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Jaqueline Galo</t>
+          <t>Felipe</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>B · Superiores</t>
+          <t>D · Sáb · Corrida</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Supino inclinado halteres + Rosca direta halteres</t>
+          <t>Aquecimento</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Peito/Bíceps</t>
-        </is>
-      </c>
-      <c r="F74" t="inlineStr">
-        <is>
-          <t>3</t>
+          <t>Corrida · aquecimento</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>5 min</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>Bi-set: sem descanso entre os dois.</t>
+          <t>Faça o aquecimento, depois SÓ o bloco da semana atual do seu ciclo, e termine no desaquecimento. A cada 4 semanas o ciclo recomeça, subindo cerca de 10%. Comece com caminhada rápida evoluindo para trote leve.</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Jaqueline Galo</t>
+          <t>Felipe</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>B · Superiores</t>
+          <t>D · Sáb · Corrida</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Abdominal remador</t>
+          <t>Semana 1 · Corrida contínua leve</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Core</t>
-        </is>
-      </c>
-      <c r="F75" t="inlineStr">
-        <is>
-          <t>3</t>
+          <t>Corrida · Semana 1</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>4-5 km</t>
         </is>
       </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t>Carga: 2 kg.</t>
+          <t>Ritmo de conversa (Z2): você consegue falar frases inteiras. Registre seu tempo total no fim.</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Jaqueline Galo</t>
+          <t>Felipe</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>C · Posterior/Glúteos</t>
+          <t>D · Sáb · Corrida</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Agachamento sumô halteres</t>
+          <t>Semana 2 · Fartlek</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Pernas/glúteos</t>
+          <t>Corrida · Semana 2</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>8 a 10</t>
+          <t>(3 min corrida + 1 min caminhada)</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>6 blocos de 3 min correndo moderado + 1 min caminhando. Registre o tempo total.</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Jaqueline Galo</t>
+          <t>Felipe</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>C · Posterior/Glúteos</t>
+          <t>D · Sáb · Corrida</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Cadeira flexora</t>
+          <t>Semana 3 · Longão leve</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Posterior de coxa</t>
-        </is>
-      </c>
-      <c r="F77" t="inlineStr">
-        <is>
-          <t>3</t>
+          <t>Corrida · Semana 3</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>15/12/10</t>
+          <t>5-6 km</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>Progressão de carga ao longo das séries.</t>
+          <t>Contínuo em Z2, sem pressa, construindo resistência. Registre seu tempo.</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Jaqueline Galo</t>
+          <t>Felipe</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>C · Posterior/Glúteos</t>
+          <t>D · Sáb · Corrida</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Glúteo chute no pulley</t>
+          <t>Semana 4 · Progressiva</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Glúteos</t>
-        </is>
-      </c>
-      <c r="F78" t="inlineStr">
-        <is>
-          <t>3</t>
+          <t>Corrida · Semana 4</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>5 km</t>
+        </is>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>Comece leve e termine o último km mais forte (limiar leve). Registre seu tempo.</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Jaqueline Galo</t>
+          <t>Felipe</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>C · Posterior/Glúteos</t>
+          <t>D · Sáb · Corrida</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Cadeira abdutora</t>
+          <t>Desaquecimento</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Glúteos · abdutores</t>
-        </is>
-      </c>
-      <c r="F79" t="inlineStr">
-        <is>
-          <t>3</t>
+          <t>Corrida · volta à calma</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>5 min</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>Trote bem leve até virar caminhada, depois alongue panturrilha, posterior e quadril.</t>
         </is>
       </c>
     </row>
@@ -4264,27 +4334,32 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>C · Posterior/Glúteos</t>
+          <t>A · Quadríceps</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Escada intervalada</t>
+          <t>Agachamento cálice</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Cardio</t>
+          <t>Quadríceps</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>3</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>2 min leve / 2 min forte × 6</t>
+          <t>15</t>
         </is>
       </c>
     </row>
@@ -4296,22 +4371,22 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>D · Circuito Full Body</t>
+          <t>A · Quadríceps</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Flexão de braço de joelhos</t>
+          <t>Afundo alternado no step</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Peito/Core</t>
+          <t>Pernas/glúteos</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -4321,12 +4396,7 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="I81" t="inlineStr">
-        <is>
-          <t>Circuito: repetir os 5 exercícios em sequência, 3 voltas — 30s de descanso entre exercícios e 2 min entre as voltas. Sem carga (peso do corpo).</t>
+          <t>10</t>
         </is>
       </c>
     </row>
@@ -4338,32 +4408,37 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>D · Circuito Full Body</t>
+          <t>A · Quadríceps</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Step-up no box</t>
+          <t>Cadeira extensora</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Pernas/glúteos</t>
+          <t>Quadríceps</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>10 cada perna</t>
+          <t>15/12/10/08</t>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>Progressão de carga ao longo das séries.</t>
         </is>
       </c>
     </row>
@@ -4375,22 +4450,22 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>D · Circuito Full Body</t>
+          <t>A · Quadríceps</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Senta e levanta com halteres no box</t>
+          <t>Leg press 45°</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Pernas/glúteos</t>
+          <t>Pernas</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
@@ -4401,6 +4476,11 @@
       <c r="G83" t="inlineStr">
         <is>
           <t>15</t>
+        </is>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>Descida lenta (controlada).</t>
         </is>
       </c>
     </row>
@@ -4412,17 +4492,17 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>D · Circuito Full Body</t>
+          <t>A · Quadríceps</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Mountain climber no box</t>
+          <t>Escada</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
@@ -4430,14 +4510,9 @@
           <t>Cardio</t>
         </is>
       </c>
-      <c r="F84" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>40s</t>
+          <t>15 min</t>
         </is>
       </c>
     </row>
@@ -4449,175 +4524,190 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>D · Circuito Full Body</t>
+          <t>B · Superiores</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Abdominal curto no solo</t>
+          <t>Puxador costas no graviton + Desenvolvimento halteres fechado</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Core</t>
+          <t>Costas/Ombro</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>máximo / 10</t>
+        </is>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>Bi-set: sem descanso entre os dois — puxador no graviton até o máximo, seguido de desenvolvimento com halteres fechado (10 reps).</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Lara</t>
+          <t>Jaqueline Galo</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>A · Tiros longos na esteira + core</t>
+          <t>B · Superiores</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Esteira — aquecimento progressivo</t>
+          <t>Pulldown barra reta (pulley) + Tríceps pulley</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Cardio · aquecimento</t>
+          <t>Costas/Tríceps</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>3</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>10 min</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>Comece em caminhada e aumente o ritmo aos poucos até um trote confortável, preparando o corpo para os tiros.</t>
+          <t>Bi-set: sem descanso entre os dois.</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Lara</t>
+          <t>Jaqueline Galo</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>A · Tiros longos na esteira + core</t>
+          <t>B · Superiores</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Esteira — tiros de 800m</t>
+          <t>Supino inclinado halteres + Rosca direta halteres</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Cardio · intervalado</t>
+          <t>Peito/Bíceps</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>800m forte</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>Cada tiro de 800m em ritmo forte, bem acima do confortável. Recuperação de 2–3 min em caminhada entre os tiros. Repita 4x.</t>
+          <t>Bi-set: sem descanso entre os dois.</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Lara</t>
+          <t>Jaqueline Galo</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>A · Tiros longos na esteira + core</t>
+          <t>B · Superiores</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Esteira — desaquecimento</t>
+          <t>Abdominal remador</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Cardio · desaquecimento</t>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>3</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>5 min</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>Trote leve reduzindo o ritmo aos poucos. Finalize com alongamento de pernas.</t>
+          <t>Carga: 2 kg.</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Lara</t>
+          <t>Jaqueline Galo</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>A · Tiros longos na esteira + core</t>
+          <t>C · Posterior/Glúteos</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Prancha abdominal</t>
+          <t>Agachamento sumô halteres</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Core</t>
+          <t>Pernas/glúteos</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
@@ -4627,390 +4717,345 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>1 min</t>
-        </is>
-      </c>
-      <c r="I89" t="inlineStr">
-        <is>
-          <t>Corpo alinhado da cabeça ao calcanhar, abdômen contraído.</t>
+          <t>8 a 10</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Lara</t>
+          <t>Jaqueline Galo</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>A · Tiros longos na esteira + core</t>
+          <t>C · Posterior/Glúteos</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Abdominal oblíquo (bicicleta)</t>
+          <t>Cadeira flexora</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Core · oblíquos</t>
+          <t>Posterior de coxa</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>15/12/10</t>
         </is>
       </c>
       <c r="I90" t="inlineStr">
         <is>
-          <t>Alterne cotovelo–joelho oposto, movimento controlado, sem puxar o pescoço.</t>
+          <t>Progressão de carga ao longo das séries.</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Lara</t>
+          <t>Jaqueline Galo</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>B · Inferiores</t>
+          <t>C · Posterior/Glúteos</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Leg press horizontal</t>
+          <t>Glúteo chute no pulley</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>Pernas · principal</t>
+          <t>Glúteos</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>15/12/10/08</t>
-        </is>
-      </c>
-      <c r="I91" t="inlineStr">
-        <is>
-          <t>Progressão de carga ao longo das séries (pirâmide): aumenta a carga e diminui as reps a cada série.</t>
+          <t>15</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Lara</t>
+          <t>Jaqueline Galo</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>B · Inferiores</t>
+          <t>C · Posterior/Glúteos</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Cadeira extensora</t>
+          <t>Cadeira abdutora</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Quadríceps</t>
+          <t>Glúteos · abdutores</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="I92" t="inlineStr">
-        <is>
-          <t>Movimento controlado, sem dar impulso; segure meio segundo no topo.</t>
+          <t>15</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Lara</t>
+          <t>Jaqueline Galo</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>B · Inferiores</t>
+          <t>C · Posterior/Glúteos</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Cadeira flexora</t>
+          <t>Escada intervalada</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Posterior de coxa</t>
-        </is>
-      </c>
-      <c r="F93" t="inlineStr">
-        <is>
-          <t>4</t>
+          <t>Cardio</t>
         </is>
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="I93" t="inlineStr">
-        <is>
-          <t>Movimento controlado, segurar 1s na contração.</t>
+          <t>2 min leve / 2 min forte × 6</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Lara</t>
+          <t>Jaqueline Galo</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>B · Inferiores</t>
+          <t>D · Circuito Full Body</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Panturrilha em pé na máquina</t>
+          <t>Flexão de braço de joelhos</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>Panturrilha · tríceps sural</t>
+          <t>Peito/Core</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I94" t="inlineStr">
         <is>
-          <t>Amplitude total, subir bem no topo e segurar 1s.</t>
+          <t>Circuito: repetir os 5 exercícios em sequência, 3 voltas — 30s de descanso entre exercícios e 2 min entre as voltas. Sem carga (peso do corpo).</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Lara</t>
+          <t>Jaqueline Galo</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>B · Inferiores</t>
+          <t>D · Circuito Full Body</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Bike — HIIT</t>
+          <t>Step-up no box</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>Cardio · intervalado</t>
+          <t>Pernas/glúteos</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>3 min pesado + 2 min devagar</t>
-        </is>
-      </c>
-      <c r="I95" t="inlineStr">
-        <is>
-          <t>6 tiros: 3 min em ritmo pesado + 2 min devagar sem carga (recuperação ativa). Repita os 6 blocos (~30 min no total).</t>
+          <t>10 cada perna</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Lara</t>
+          <t>Jaqueline Galo</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>C · Circuito de braço + tiros</t>
+          <t>D · Circuito Full Body</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Puxador frente delta + Rosca direta (bi-set)</t>
+          <t>Senta e levanta com halteres no box</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>Dorsais · bíceps</t>
+          <t>Pernas/glúteos</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>15 / 20</t>
-        </is>
-      </c>
-      <c r="I96" t="inlineStr">
-        <is>
-          <t>Bi-set sem descanso: puxador frente com pegada delta 15 reps, emenda rosca direta com halteres 20 reps. Descanse e repita 4x.</t>
+          <t>15</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Lara</t>
+          <t>Jaqueline Galo</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>C · Circuito de braço + tiros</t>
+          <t>D · Circuito Full Body</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Esteira — 800m</t>
+          <t>Mountain climber no box</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>Cardio · intervalado</t>
+          <t>Cardio</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>800m forte</t>
-        </is>
-      </c>
-      <c r="I97" t="inlineStr">
-        <is>
-          <t>Tiro de 800m em ritmo forte logo depois do bi-set.</t>
+          <t>40s</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Lara</t>
+          <t>Jaqueline Galo</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>C · Circuito de braço + tiros</t>
+          <t>D · Circuito Full Body</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Remada sentada + Desenvolvimento com halteres em pé (bi-set)</t>
+          <t>Abdominal curto no solo</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>Costas · ombro</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>15 cada</t>
-        </is>
-      </c>
-      <c r="I98" t="inlineStr">
-        <is>
-          <t>Bi-set sem descanso: remada sentada 15 reps, emenda desenvolvimento com halteres em pé 15 reps. Repita 4x.</t>
+          <t>20</t>
         </is>
       </c>
     </row>
@@ -5022,37 +5067,32 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>C · Circuito de braço + tiros</t>
+          <t>A · Tiros longos na esteira + core</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Esteira — 800m</t>
+          <t>Esteira — aquecimento progressivo</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Cardio · intervalado</t>
-        </is>
-      </c>
-      <c r="F99" t="inlineStr">
-        <is>
-          <t>1</t>
+          <t>Cardio · aquecimento</t>
         </is>
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>800m forte</t>
+          <t>10 min</t>
         </is>
       </c>
       <c r="I99" t="inlineStr">
         <is>
-          <t>Tiro de 800m em ritmo forte.</t>
+          <t>Comece em caminhada e aumente o ritmo aos poucos até um trote confortável, preparando o corpo para os tiros.</t>
         </is>
       </c>
     </row>
@@ -5064,22 +5104,22 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>C · Circuito de braço + tiros</t>
+          <t>A · Tiros longos na esteira + core</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Supino sentado na máquina + Tríceps francês com halteres (bi-set)</t>
+          <t>Esteira — tiros de 800m</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>Peitoral · tríceps</t>
+          <t>Cardio · intervalado</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
@@ -5089,12 +5129,12 @@
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>15 cada</t>
+          <t>800m forte</t>
         </is>
       </c>
       <c r="I100" t="inlineStr">
         <is>
-          <t>Bi-set sem descanso: supino sentado na máquina 15 reps, emenda tríceps francês com halteres 15 reps. Repita 4x.</t>
+          <t>Cada tiro de 800m em ritmo forte, bem acima do confortável. Recuperação de 2–3 min em caminhada entre os tiros. Repita 4x.</t>
         </is>
       </c>
     </row>
@@ -5106,37 +5146,32 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>C · Circuito de braço + tiros</t>
+          <t>A · Tiros longos na esteira + core</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Esteira — 800m</t>
+          <t>Esteira — desaquecimento</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>Cardio · intervalado</t>
-        </is>
-      </c>
-      <c r="F101" t="inlineStr">
-        <is>
-          <t>1</t>
+          <t>Cardio · desaquecimento</t>
         </is>
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>800m forte</t>
+          <t>5 min</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
         <is>
-          <t>Último tiro de 800m em ritmo forte.</t>
+          <t>Trote leve reduzindo o ritmo aos poucos. Finalize com alongamento de pernas.</t>
         </is>
       </c>
     </row>
@@ -5148,17 +5183,17 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>C · Circuito de braço + tiros</t>
+          <t>A · Tiros longos na esteira + core</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>Abdominal curto com peso</t>
+          <t>Prancha abdominal</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
@@ -5173,12 +5208,12 @@
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>1 min</t>
         </is>
       </c>
       <c r="I102" t="inlineStr">
         <is>
-          <t>Segure o peso no peito, contraia o abdômen no topo sem puxar o pescoço.</t>
+          <t>Corpo alinhado da cabeça ao calcanhar, abdômen contraído.</t>
         </is>
       </c>
     </row>
@@ -5190,32 +5225,37 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>D · Corrida + glúteos</t>
+          <t>A · Tiros longos na esteira + core</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>Esteira — corrida contínua</t>
+          <t>Abdominal oblíquo (bicicleta)</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Cardio · aeróbico</t>
+          <t>Core · oblíquos</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>4</t>
         </is>
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>3 km sem parar</t>
+          <t>20</t>
         </is>
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>Ritmo moderado e constante, sem pausa. Respiração controlada — dá pra manter conversa curta.</t>
+          <t>Alterne cotovelo–joelho oposto, movimento controlado, sem puxar o pescoço.</t>
         </is>
       </c>
     </row>
@@ -5227,22 +5267,22 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>D · Corrida + glúteos</t>
+          <t>B · Inferiores</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>Agachamento sumô com kettlebell</t>
+          <t>Leg press horizontal</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Glúteos/pernas · principal</t>
+          <t>Pernas · principal</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
@@ -5252,12 +5292,12 @@
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>15/12/10/08</t>
         </is>
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>Pés afastados e pontas abertas; desça mantendo o tronco ereto e o peso no calcanhar.</t>
+          <t>Progressão de carga ao longo das séries (pirâmide): aumenta a carga e diminui as reps a cada série.</t>
         </is>
       </c>
     </row>
@@ -5269,22 +5309,22 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>D · Corrida + glúteos</t>
+          <t>B · Inferiores</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Cadeira abdutora</t>
+          <t>Cadeira extensora</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>Glúteos · abdutores</t>
+          <t>Quadríceps</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
@@ -5294,12 +5334,12 @@
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>20</t>
         </is>
       </c>
       <c r="I105" t="inlineStr">
         <is>
-          <t>Abrir as pernas com controle, sem jogar o tronco para trás.</t>
+          <t>Movimento controlado, sem dar impulso; segure meio segundo no topo.</t>
         </is>
       </c>
     </row>
@@ -5311,22 +5351,22 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>D · Corrida + glúteos</t>
+          <t>B · Inferiores</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>Glúteo coice na polia</t>
+          <t>Cadeira flexora</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>Glúteos</t>
+          <t>Posterior de coxa</t>
         </is>
       </c>
       <c r="F106" t="inlineStr">
@@ -5336,12 +5376,12 @@
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I106" t="inlineStr">
         <is>
-          <t>Movimento controlado; contraia o glúteo no topo sem hiperestender a lombar.</t>
+          <t>Movimento controlado, segurar 1s na contração.</t>
         </is>
       </c>
     </row>
@@ -5353,22 +5393,22 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>D · Corrida + glúteos</t>
+          <t>B · Inferiores</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>Prancha abdominal</t>
+          <t>Panturrilha em pé na máquina</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>Core</t>
+          <t>Panturrilha · tríceps sural</t>
         </is>
       </c>
       <c r="F107" t="inlineStr">
@@ -5378,82 +5418,81 @@
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>1 min</t>
+          <t>20</t>
         </is>
       </c>
       <c r="I107" t="inlineStr">
         <is>
-          <t>Corpo alinhado da cabeça ao calcanhar, abdômen contraído.</t>
+          <t>Amplitude total, subir bem no topo e segurar 1s.</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Marina Barbato</t>
+          <t>Lara</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>A · Seg · Quadríceps</t>
+          <t>B · Inferiores</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>Agachamento livre (ativação)</t>
+          <t>Bike — HIIT</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>Quadríceps</t>
+          <t>Cardio · intervalado</t>
         </is>
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>6</t>
         </is>
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="H108" t="inlineStr"/>
+          <t>3 min pesado + 2 min devagar</t>
+        </is>
+      </c>
       <c r="I108" t="inlineStr">
         <is>
-          <t>Descida lenta (excêntrica controlada) — séries de ativação antes da carga.</t>
+          <t>6 tiros: 3 min em ritmo pesado + 2 min devagar sem carga (recuperação ativa). Repita os 6 blocos (~30 min no total).</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Marina Barbato</t>
+          <t>Lara</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>A · Seg · Quadríceps</t>
+          <t>C · Circuito de braço + tiros</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>Agachamento livre (carga)</t>
+          <t>Puxador frente delta + Rosca direta (bi-set)</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>Quadríceps</t>
+          <t>Dorsais · bíceps</t>
         </is>
       </c>
       <c r="F109" t="inlineStr">
@@ -5463,83 +5502,81 @@
       </c>
       <c r="G109" t="inlineStr">
         <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="H109" t="inlineStr"/>
+          <t>15 / 20</t>
+        </is>
+      </c>
       <c r="I109" t="inlineStr">
         <is>
-          <t>Séries de trabalho, na sequência das 2 séries de ativação.</t>
+          <t>Bi-set sem descanso: puxador frente com pegada delta 15 reps, emenda rosca direta com halteres 20 reps. Descanse e repita 4x.</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Marina Barbato</t>
+          <t>Lara</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>A · Seg · Quadríceps</t>
+          <t>C · Circuito de braço + tiros</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>Leg press 45°</t>
+          <t>Esteira — 800m</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>Quadríceps</t>
+          <t>Cardio · intervalado</t>
         </is>
       </c>
       <c r="F110" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G110" t="inlineStr">
         <is>
-          <t>20/15/12/10/8</t>
-        </is>
-      </c>
-      <c r="H110" t="inlineStr"/>
+          <t>800m forte</t>
+        </is>
+      </c>
       <c r="I110" t="inlineStr">
         <is>
-          <t>Progressão de carga a cada série.</t>
+          <t>Tiro de 800m em ritmo forte logo depois do bi-set.</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Marina Barbato</t>
+          <t>Lara</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>A · Seg · Quadríceps</t>
+          <t>C · Circuito de braço + tiros</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>Cadeira extensora</t>
+          <t>Remada sentada + Desenvolvimento com halteres em pé (bi-set)</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>Quadríceps</t>
+          <t>Costas · ombro</t>
         </is>
       </c>
       <c r="F111" t="inlineStr">
@@ -5549,78 +5586,81 @@
       </c>
       <c r="G111" t="inlineStr">
         <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="H111" t="inlineStr"/>
+          <t>15 cada</t>
+        </is>
+      </c>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>Bi-set sem descanso: remada sentada 15 reps, emenda desenvolvimento com halteres em pé 15 reps. Repita 4x.</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>Marina Barbato</t>
+          <t>Lara</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>A · Seg · Quadríceps</t>
+          <t>C · Circuito de braço + tiros</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>Cadeira extensora</t>
+          <t>Esteira — 800m</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>Quadríceps</t>
+          <t>Cardio · intervalado</t>
         </is>
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G112" t="inlineStr">
         <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="H112" t="inlineStr"/>
+          <t>800m forte</t>
+        </is>
+      </c>
       <c r="I112" t="inlineStr">
         <is>
-          <t>Segundo bloco — aumentar a carga.</t>
+          <t>Tiro de 800m em ritmo forte.</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>Marina Barbato</t>
+          <t>Lara</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>A · Seg · Quadríceps</t>
+          <t>C · Circuito de braço + tiros</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>Panturrilha em pé</t>
+          <t>Supino sentado na máquina + Tríceps francês com halteres (bi-set)</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>Panturrilha</t>
+          <t>Peitoral · tríceps</t>
         </is>
       </c>
       <c r="F113" t="inlineStr">
@@ -5630,78 +5670,81 @@
       </c>
       <c r="G113" t="inlineStr">
         <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="H113" t="inlineStr"/>
+          <t>15 cada</t>
+        </is>
+      </c>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>Bi-set sem descanso: supino sentado na máquina 15 reps, emenda tríceps francês com halteres 15 reps. Repita 4x.</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>Marina Barbato</t>
+          <t>Lara</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>B · Ter · Dorsal</t>
+          <t>C · Circuito de braço + tiros</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>Remada sentada pulley</t>
+          <t>Esteira — 800m</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>Dorsal</t>
+          <t>Cardio · intervalado</t>
         </is>
       </c>
       <c r="F114" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G114" t="inlineStr">
         <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="H114" t="inlineStr"/>
+          <t>800m forte</t>
+        </is>
+      </c>
       <c r="I114" t="inlineStr">
         <is>
-          <t>Bi-set com a rosca direta com halteres (próximo exercício), sem descanso entre eles.</t>
+          <t>Último tiro de 800m em ritmo forte.</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>Marina Barbato</t>
+          <t>Lara</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>B · Ter · Dorsal</t>
+          <t>C · Circuito de braço + tiros</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>Rosca direta halteres</t>
+          <t>Abdominal curto com peso</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>Bíceps</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="F115" t="inlineStr">
@@ -5711,122 +5754,118 @@
       </c>
       <c r="G115" t="inlineStr">
         <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="H115" t="inlineStr"/>
+          <t>15</t>
+        </is>
+      </c>
       <c r="I115" t="inlineStr">
         <is>
-          <t>Bi-set com a remada sentada pulley (exercício anterior).</t>
+          <t>Segure o peso no peito, contraia o abdômen no topo sem puxar o pescoço.</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>Marina Barbato</t>
+          <t>Lara</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>B · Ter · Dorsal</t>
+          <t>D · Corrida + glúteos</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>Puxador aberto pulley</t>
+          <t>Esteira — corrida contínua</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>Dorsal</t>
-        </is>
-      </c>
-      <c r="F116" t="inlineStr">
-        <is>
-          <t>4</t>
+          <t>Cardio · aeróbico</t>
         </is>
       </c>
       <c r="G116" t="inlineStr">
         <is>
-          <t>15/12/10/8</t>
-        </is>
-      </c>
-      <c r="H116" t="inlineStr"/>
+          <t>3 km sem parar</t>
+        </is>
+      </c>
       <c r="I116" t="inlineStr">
         <is>
-          <t>Progressão de carga a cada série.</t>
+          <t>Ritmo moderado e constante, sem pausa. Respiração controlada — dá pra manter conversa curta.</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>Marina Barbato</t>
+          <t>Lara</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>B · Ter · Dorsal</t>
+          <t>D · Corrida + glúteos</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>Remo aeróbico</t>
+          <t>Agachamento sumô com kettlebell</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>Cardio</t>
-        </is>
-      </c>
-      <c r="F117" t="inlineStr"/>
+          <t>Glúteos/pernas · principal</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
       <c r="G117" t="inlineStr">
         <is>
-          <t>10 min</t>
-        </is>
-      </c>
-      <c r="H117" t="inlineStr"/>
+          <t>15</t>
+        </is>
+      </c>
       <c r="I117" t="inlineStr">
         <is>
-          <t>Ritmo moderado-intenso.</t>
+          <t>Pés afastados e pontas abertas; desça mantendo o tronco ereto e o peso no calcanhar.</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>Marina Barbato</t>
+          <t>Lara</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>B · Ter · Dorsal</t>
+          <t>D · Corrida + glúteos</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>Banco romano</t>
+          <t>Cadeira abdutora</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>Lombar/Posterior</t>
+          <t>Glúteos · abdutores</t>
         </is>
       </c>
       <c r="F118" t="inlineStr">
@@ -5839,37 +5878,36 @@
           <t>15</t>
         </is>
       </c>
-      <c r="H118" t="inlineStr"/>
       <c r="I118" t="inlineStr">
         <is>
-          <t>Descida lenta (excêntrica controlada).</t>
+          <t>Abrir as pernas com controle, sem jogar o tronco para trás.</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>Marina Barbato</t>
+          <t>Lara</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>C · Qua · Posterior de coxa</t>
+          <t>D · Corrida + glúteos</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>Mesa flexora</t>
+          <t>Glúteo coice na polia</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>Posterior de coxa</t>
+          <t>Glúteos</t>
         </is>
       </c>
       <c r="F119" t="inlineStr">
@@ -5879,35 +5917,39 @@
       </c>
       <c r="G119" t="inlineStr">
         <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="H119" t="inlineStr"/>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="I119" t="inlineStr">
+        <is>
+          <t>Movimento controlado; contraia o glúteo no topo sem hiperestender a lombar.</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>Marina Barbato</t>
+          <t>Lara</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>C · Qua · Posterior de coxa</t>
+          <t>D · Corrida + glúteos</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>Mesa flexora</t>
+          <t>Prancha abdominal</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>Posterior de coxa</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
@@ -5917,13 +5959,12 @@
       </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="H120" t="inlineStr"/>
+          <t>1 min</t>
+        </is>
+      </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>Segundo bloco — aumentar a carga.</t>
+          <t>Corpo alinhado da cabeça ao calcanhar, abdômen contraído.</t>
         </is>
       </c>
     </row>
@@ -5935,35 +5976,39 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>C · Qua · Posterior de coxa</t>
+          <t>A · Seg · Quadríceps</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>Flexor de joelhos em pé</t>
+          <t>Agachamento livre (ativação)</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>Posterior de coxa</t>
+          <t>Quadríceps</t>
         </is>
       </c>
       <c r="F121" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G121" t="inlineStr">
         <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="H121" t="inlineStr"/>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="I121" t="inlineStr">
+        <is>
+          <t>Descida lenta (excêntrica controlada) — séries de ativação antes da carga.</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -5973,22 +6018,22 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>C · Qua · Posterior de coxa</t>
+          <t>A · Seg · Quadríceps</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>Stiff halteres</t>
+          <t>Agachamento livre (carga)</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>Posterior de coxa/Glúteo</t>
+          <t>Quadríceps</t>
         </is>
       </c>
       <c r="F122" t="inlineStr">
@@ -5998,10 +6043,14 @@
       </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="H122" t="inlineStr"/>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>Séries de trabalho, na sequência das 2 séries de ativação.</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -6011,35 +6060,39 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>C · Qua · Posterior de coxa</t>
+          <t>A · Seg · Quadríceps</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>Abdominal máquina</t>
+          <t>Leg press 45°</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>Abdômen</t>
+          <t>Quadríceps</t>
         </is>
       </c>
       <c r="F123" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="G123" t="inlineStr">
         <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="H123" t="inlineStr"/>
+          <t>20/15/12/10/8</t>
+        </is>
+      </c>
+      <c r="I123" t="inlineStr">
+        <is>
+          <t>Progressão de carga a cada série.</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -6049,22 +6102,22 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>D · Qui · Ombro, Tríceps e Bíceps</t>
+          <t>A · Seg · Quadríceps</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>Manguito rotador (elástico ou pulley)</t>
+          <t>Cadeira extensora</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>Ombro</t>
+          <t>Quadríceps</t>
         </is>
       </c>
       <c r="F124" t="inlineStr">
@@ -6074,13 +6127,7 @@
       </c>
       <c r="G124" t="inlineStr">
         <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="H124" t="inlineStr"/>
-      <c r="I124" t="inlineStr">
-        <is>
-          <t>Ativação do manguito rotador antes da carga.</t>
+          <t>20</t>
         </is>
       </c>
     </row>
@@ -6092,22 +6139,22 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>D · Qui · Ombro, Tríceps e Bíceps</t>
+          <t>A · Seg · Quadríceps</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>Elevação lateral halteres</t>
+          <t>Cadeira extensora</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>Ombro</t>
+          <t>Quadríceps</t>
         </is>
       </c>
       <c r="F125" t="inlineStr">
@@ -6117,10 +6164,14 @@
       </c>
       <c r="G125" t="inlineStr">
         <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="H125" t="inlineStr"/>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>Segundo bloco — aumentar a carga.</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -6130,22 +6181,22 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>D · Qui · Ombro, Tríceps e Bíceps</t>
+          <t>A · Seg · Quadríceps</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>Elevação lateral no pulley</t>
+          <t>Panturrilha em pé</t>
         </is>
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>Ombro</t>
+          <t>Panturrilha</t>
         </is>
       </c>
       <c r="F126" t="inlineStr">
@@ -6155,10 +6206,9 @@
       </c>
       <c r="G126" t="inlineStr">
         <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="H126" t="inlineStr"/>
+          <t>20</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -6168,22 +6218,22 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>D · Qui · Ombro, Tríceps e Bíceps</t>
+          <t>B · Ter · Dorsal</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>Desenvolvimento fechado halteres</t>
+          <t>Remada sentada pulley</t>
         </is>
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>Ombro</t>
+          <t>Dorsal</t>
         </is>
       </c>
       <c r="F127" t="inlineStr">
@@ -6193,10 +6243,14 @@
       </c>
       <c r="G127" t="inlineStr">
         <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="H127" t="inlineStr"/>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="I127" t="inlineStr">
+        <is>
+          <t>Bi-set com a rosca direta com halteres (próximo exercício), sem descanso entre eles.</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -6206,35 +6260,39 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>D · Qui · Ombro, Tríceps e Bíceps</t>
+          <t>B · Ter · Dorsal</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>Tríceps pulley corda</t>
+          <t>Rosca direta halteres</t>
         </is>
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>Tríceps</t>
+          <t>Bíceps</t>
         </is>
       </c>
       <c r="F128" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G128" t="inlineStr">
         <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="H128" t="inlineStr"/>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="I128" t="inlineStr">
+        <is>
+          <t>Bi-set com a remada sentada pulley (exercício anterior).</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -6244,22 +6302,22 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>E · Sex · Glúteos</t>
+          <t>B · Ter · Dorsal</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>Supino sentada</t>
+          <t>Puxador aberto pulley</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>Glúteo</t>
+          <t>Dorsal</t>
         </is>
       </c>
       <c r="F129" t="inlineStr">
@@ -6269,13 +6327,12 @@
       </c>
       <c r="G129" t="inlineStr">
         <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="H129" t="inlineStr"/>
+          <t>15/12/10/8</t>
+        </is>
+      </c>
       <c r="I129" t="inlineStr">
         <is>
-          <t>Confirmar nome do aparelho com a Larissa.</t>
+          <t>Progressão de carga a cada série.</t>
         </is>
       </c>
     </row>
@@ -6287,35 +6344,34 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>E · Sex · Glúteos</t>
+          <t>B · Ter · Dorsal</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>Cadeira abdutora</t>
+          <t>Remo aeróbico</t>
         </is>
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>Glúteo médio</t>
-        </is>
-      </c>
-      <c r="F130" t="inlineStr">
-        <is>
-          <t>4</t>
+          <t>Cardio</t>
         </is>
       </c>
       <c r="G130" t="inlineStr">
         <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="H130" t="inlineStr"/>
+          <t>10 min</t>
+        </is>
+      </c>
+      <c r="I130" t="inlineStr">
+        <is>
+          <t>Ritmo moderado-intenso.</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -6325,22 +6381,22 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>E · Sex · Glúteos</t>
+          <t>B · Ter · Dorsal</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>Elevação pélvica</t>
+          <t>Banco romano</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>Glúteo</t>
+          <t>Lombar/Posterior</t>
         </is>
       </c>
       <c r="F131" t="inlineStr">
@@ -6350,10 +6406,14 @@
       </c>
       <c r="G131" t="inlineStr">
         <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="H131" t="inlineStr"/>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="I131" t="inlineStr">
+        <is>
+          <t>Descida lenta (excêntrica controlada).</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -6363,22 +6423,22 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>C</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>E · Sex · Glúteos</t>
+          <t>C · Qua · Posterior de coxa</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>Glúteo no pulley (extensão de quadril)</t>
+          <t>Mesa flexora</t>
         </is>
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>Glúteo</t>
+          <t>Posterior de coxa</t>
         </is>
       </c>
       <c r="F132" t="inlineStr">
@@ -6388,10 +6448,9 @@
       </c>
       <c r="G132" t="inlineStr">
         <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="H132" t="inlineStr"/>
+          <t>20</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -6401,35 +6460,530 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>C · Qua · Posterior de coxa</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>Mesa flexora</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>Posterior de coxa</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G133" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="I133" t="inlineStr">
+        <is>
+          <t>Segundo bloco — aumentar a carga.</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>Marina Barbato</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>C · Qua · Posterior de coxa</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>Flexor de joelhos em pé</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>Posterior de coxa</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>Marina Barbato</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>C · Qua · Posterior de coxa</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>Stiff halteres</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>Posterior de coxa/Glúteo</t>
+        </is>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G135" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>Marina Barbato</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>C · Qua · Posterior de coxa</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>Abdominal máquina</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>Abdômen</t>
+        </is>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G136" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>Marina Barbato</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>D · Qui · Ombro, Tríceps e Bíceps</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>Manguito rotador (elástico ou pulley)</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>Ombro</t>
+        </is>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G137" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="I137" t="inlineStr">
+        <is>
+          <t>Ativação do manguito rotador antes da carga.</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>Marina Barbato</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>D · Qui · Ombro, Tríceps e Bíceps</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>Elevação lateral halteres</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>Ombro</t>
+        </is>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G138" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>Marina Barbato</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>D · Qui · Ombro, Tríceps e Bíceps</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>Elevação lateral no pulley</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>Ombro</t>
+        </is>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G139" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>Marina Barbato</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>D · Qui · Ombro, Tríceps e Bíceps</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>Desenvolvimento fechado halteres</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>Ombro</t>
+        </is>
+      </c>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G140" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>Marina Barbato</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>D · Qui · Ombro, Tríceps e Bíceps</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>Tríceps pulley corda</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>Tríceps</t>
+        </is>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="G141" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>Marina Barbato</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
           <t>E</t>
         </is>
       </c>
-      <c r="C133" t="inlineStr">
+      <c r="C142" t="inlineStr">
         <is>
           <t>E · Sex · Glúteos</t>
         </is>
       </c>
-      <c r="D133" t="inlineStr">
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>Supino sentada</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>Glúteo</t>
+        </is>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G142" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="I142" t="inlineStr">
+        <is>
+          <t>Confirmar nome do aparelho com a Larissa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>Marina Barbato</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>E · Sex · Glúteos</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>Cadeira abdutora</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>Glúteo médio</t>
+        </is>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G143" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>Marina Barbato</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>E · Sex · Glúteos</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>Elevação pélvica</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>Glúteo</t>
+        </is>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G144" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>Marina Barbato</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>E · Sex · Glúteos</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>Glúteo no pulley (extensão de quadril)</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>Glúteo</t>
+        </is>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G145" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>Marina Barbato</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>E · Sex · Glúteos</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
         <is>
           <t>Glúteo — chute na máquina</t>
         </is>
       </c>
-      <c r="E133" t="inlineStr">
+      <c r="E146" t="inlineStr">
         <is>
           <t>Glúteo</t>
         </is>
       </c>
-      <c r="F133" t="inlineStr">
+      <c r="F146" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="G133" t="inlineStr">
+      <c r="G146" t="inlineStr">
         <is>
           <t>15</t>
         </is>
       </c>
-      <c r="H133" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Nilo: treino de pernas (quarta) no app
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/gerador/modelo-treinos.xlsx
+++ b/gerador/modelo-treinos.xlsx
@@ -805,7 +805,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Foco: perda de gordura e hipertrofia de peitorais · Musculação 5x (Peito/Costas/Pernas presencial/Ombros/Bíceps+Tríceps) + atividade livre</t>
+          <t>Foco: perda de gordura e hipertrofia de peitorais · Musculação 5x (Peito/Costas/Pernas/Ombros/Bíceps+Tríceps) + atividade livre</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -815,7 +815,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Ciclo com prioridade em peitoral: segunda peito, terça costas, quarta pernas (presencial comigo), quinta ombros e sexta bíceps/tríceps, com o treino de peito estruturado para máximo estímulo (bi-set e drop set). A musculação fecha o déficit calórico junto com a atividade livre, por conta do próprio Nilo (CrossFit, cardio ou o que preferir nos dias livres).</t>
+          <t>Ciclo com prioridade em peitoral: segunda peito, terça costas, quarta pernas, quinta ombros e sexta bíceps/tríceps, com o treino de peito estruturado para máximo estímulo (bi-set e drop set). A musculação fecha o déficit calórico junto com a atividade livre, por conta do próprio Nilo (CrossFit, cardio ou o que preferir nos dias livres).</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -1038,7 +1038,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J146"/>
+  <dimension ref="A1:J150"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2820,22 +2820,32 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>C · Qua · Pernas (presencial)</t>
+          <t>C · Qua · Pernas</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Treino presencial com a Larissa</t>
+          <t>Agachamento no Smith</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Pernas</t>
+          <t>Quadríceps / Glúteos</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>12/12/12/12/12</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>Treino de pernas feito presencialmente comigo. Os exercícios e cargas são passados na hora.</t>
+          <t>Progressão de carga: mantém as 12 reps e aumenta a carga a cada série.</t>
         </is>
       </c>
     </row>
@@ -2847,37 +2857,37 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>D · Qui · Ombros</t>
+          <t>C · Qua · Pernas</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Manguito rotador no pulley (rotação externa)</t>
+          <t>Leg press</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Manguito rotador</t>
+          <t>Quadríceps / Glúteos</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>12/12/12/12/12</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>Cotovelo colado ao corpo, gira o antebraço pra fora. Carga leve, movimento controlado.</t>
+          <t>Progressão de carga: mantém as 12 reps e aumenta a carga a cada série.</t>
         </is>
       </c>
     </row>
@@ -2889,37 +2899,37 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>D · Qui · Ombros</t>
+          <t>C · Qua · Pernas</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Desenvolvimento na máquina</t>
+          <t>Cadeira extensora</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Deltoide</t>
+          <t>Quadríceps</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>12/12/12/12</t>
+          <t>15/12/10</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>Progressão de carga: mantém as 12 reps e aumenta a carga a cada série.</t>
+          <t>Drop set: tudo na MESMA série, reduz a carga sem descanso (15 → 12 → 10) até a falha.</t>
         </is>
       </c>
     </row>
@@ -2931,37 +2941,37 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>D · Qui · Ombros</t>
+          <t>C · Qua · Pernas</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Elevação lateral sentado no banco</t>
+          <t>Mesa flexora</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Deltoide lateral</t>
+          <t>Posterior de coxa</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>15/12/10</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>Drop set: tudo na MESMA série, reduz a carga sem descanso (15 → 12 → 10) até a falha.</t>
+          <t>Controla a descida, sem tirar o quadril do banco.</t>
         </is>
       </c>
     </row>
@@ -2973,22 +2983,22 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>D · Qui · Ombros</t>
+          <t>C · Qua · Pernas</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Elevação frontal unilateral no pulley</t>
+          <t>Panturrilha em pé na máquina</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Deltoide anterior</t>
+          <t>Panturrilha</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -3003,7 +3013,7 @@
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>Um braço de cada vez, sobe até a altura do ombro e controla a descida.</t>
+          <t>Amplitude total: desce alongando e sobe até a ponta dos pés.</t>
         </is>
       </c>
     </row>
@@ -3025,12 +3035,12 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Abdominal na máquina</t>
+          <t>Manguito rotador no pulley (rotação externa)</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Core</t>
+          <t>Manguito rotador</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -3045,7 +3055,7 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>Contrai o abdômen, sem puxar com os braços.</t>
+          <t>Cotovelo colado ao corpo, gira o antebraço pra fora. Carga leve, movimento controlado.</t>
         </is>
       </c>
     </row>
@@ -3057,22 +3067,22 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>E · Sex · Bíceps e Tríceps</t>
+          <t>D · Qui · Ombros</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Rosca direta na máquina</t>
+          <t>Desenvolvimento na máquina</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Bíceps</t>
+          <t>Deltoide</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -3099,37 +3109,37 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>E · Sex · Bíceps e Tríceps</t>
+          <t>D · Qui · Ombros</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Tríceps inverso no pulley (barra reta)</t>
+          <t>Elevação lateral sentado no banco</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Tríceps</t>
+          <t>Deltoide lateral</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>15/12/12/12</t>
+          <t>15/12/10</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>Pegada inversa (palmas pra cima). Progressão de carga ao longo das séries.</t>
+          <t>Drop set: tudo na MESMA série, reduz a carga sem descanso (15 → 12 → 10) até a falha.</t>
         </is>
       </c>
     </row>
@@ -3141,37 +3151,37 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>E · Sex · Bíceps e Tríceps</t>
+          <t>D · Qui · Ombros</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Rosca scott na máquina</t>
+          <t>Elevação frontal unilateral no pulley</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Bíceps</t>
+          <t>Deltoide anterior</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>15/12/10</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>Drop set: tudo na MESMA série, reduz a carga sem descanso (15 → 12 → 10) até a falha.</t>
+          <t>Um braço de cada vez, sobe até a altura do ombro e controla a descida.</t>
         </is>
       </c>
     </row>
@@ -3183,37 +3193,37 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>E · Sex · Bíceps e Tríceps</t>
+          <t>D · Qui · Ombros</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Tríceps no pulley com corda</t>
+          <t>Abdominal na máquina</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Tríceps</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>15/12/10</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>Drop set: tudo na MESMA série, reduz a carga sem descanso (15 → 12 → 10) até a falha.</t>
+          <t>Contrai o abdômen, sem puxar com os braços.</t>
         </is>
       </c>
     </row>
@@ -3235,12 +3245,12 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Abdominal na máquina</t>
+          <t>Rosca direta na máquina</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Core</t>
+          <t>Bíceps</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -3250,39 +3260,39 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>12/12/12/12</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>Contrai o abdômen, sem puxar com os braços.</t>
+          <t>Progressão de carga: mantém as 12 reps e aumenta a carga a cada série.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Felipe</t>
+          <t>Nilo Sheeny</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>E</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>A · Ter · Peito</t>
+          <t>E · Sex · Bíceps e Tríceps</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Supino na máquina (chest press)</t>
+          <t>Tríceps inverso no pulley (barra reta)</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Peitoral · principal</t>
+          <t>Tríceps</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -3292,81 +3302,81 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>12/10/8/8</t>
+          <t>15/12/12/12</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>Progressão de carga ao longo das séries. Empurra controlado, sem travar o cotovelo no fim.</t>
+          <t>Pegada inversa (palmas pra cima). Progressão de carga ao longo das séries.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Felipe</t>
+          <t>Nilo Sheeny</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>E</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>A · Ter · Peito</t>
+          <t>E · Sex · Bíceps e Tríceps</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Supino inclinado com halteres</t>
+          <t>Rosca scott na máquina</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Peitoral</t>
+          <t>Bíceps</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>15/12/10</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>Progressão de carga: aumente o peso a cada série mantendo a técnica.</t>
+          <t>Drop set: tudo na MESMA série, reduz a carga sem descanso (15 → 12 → 10) até a falha.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Felipe</t>
+          <t>Nilo Sheeny</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>E</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>A · Ter · Peito</t>
+          <t>E · Sex · Bíceps e Tríceps</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Crucifixo na máquina (voador)</t>
+          <t>Tríceps no pulley com corda</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Peitoral</t>
+          <t>Tríceps</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -3376,54 +3386,54 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>15/12/10</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>Abre bem e segura 1 seg na contração.</t>
+          <t>Drop set: tudo na MESMA série, reduz a carga sem descanso (15 → 12 → 10) até a falha.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Felipe</t>
+          <t>Nilo Sheeny</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>E</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>A · Ter · Peito</t>
+          <t>E · Sex · Bíceps e Tríceps</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Crossover na polia</t>
+          <t>Abdominal na máquina</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Peitoral</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>15/12/10</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>Drop set: tudo na MESMA série, reduz a carga sem descanso (15 → 12 → 10) até a falha.</t>
+          <t>Contrai o abdômen, sem puxar com os braços.</t>
         </is>
       </c>
     </row>
@@ -3445,27 +3455,27 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Tríceps na corda</t>
+          <t>Supino na máquina (chest press)</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Tríceps</t>
+          <t>Peitoral · principal</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>12/10/8/8</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>Cotovelos fixos junto ao corpo, abre bem no fim.</t>
+          <t>Progressão de carga ao longo das séries. Empurra controlado, sem travar o cotovelo no fim.</t>
         </is>
       </c>
     </row>
@@ -3487,27 +3497,27 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Tríceps testa</t>
+          <t>Supino inclinado com halteres</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Tríceps</t>
+          <t>Peitoral</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>15/12/10</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>Drop set: tudo na MESMA série, reduz a carga sem descanso (15 → 12 → 10) até a falha.</t>
+          <t>Progressão de carga: aumente o peso a cada série mantendo a técnica.</t>
         </is>
       </c>
     </row>
@@ -3519,37 +3529,37 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>B · Qui · Costas</t>
+          <t>A · Ter · Peito</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Barra fixa ou puxada alta (pegada aberta)</t>
+          <t>Crucifixo na máquina (voador)</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Costas · principal</t>
+          <t>Peitoral</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>12/10/8/8</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>Progressão de carga ao longo das séries.</t>
+          <t>Abre bem e segura 1 seg na contração.</t>
         </is>
       </c>
     </row>
@@ -3561,37 +3571,37 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>B · Qui · Costas</t>
+          <t>A · Ter · Peito</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Remada sentada na máquina (pegada neutra)</t>
+          <t>Crossover na polia</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Costas</t>
+          <t>Peitoral</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>12/10/10/08</t>
+          <t>15/12/10</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>Progressão de carga. Controla a fase negativa.</t>
+          <t>Drop set: tudo na MESMA série, reduz a carga sem descanso (15 → 12 → 10) até a falha.</t>
         </is>
       </c>
     </row>
@@ -3603,22 +3613,22 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>B · Qui · Costas</t>
+          <t>A · Ter · Peito</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Remada cavalinho (T-bar)</t>
+          <t>Tríceps na corda</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Costas</t>
+          <t>Tríceps</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -3628,12 +3638,12 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>10-12</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>Peito apoiado, puxa com os cotovelos.</t>
+          <t>Cotovelos fixos junto ao corpo, abre bem no fim.</t>
         </is>
       </c>
     </row>
@@ -3645,22 +3655,22 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>B · Qui · Costas</t>
+          <t>A · Ter · Peito</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Puxada com triângulo (pegada neutra)</t>
+          <t>Tríceps testa</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Costas</t>
+          <t>Tríceps</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
@@ -3670,12 +3680,12 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>15/12/10</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>Leva o triângulo ao peito, escápulas pra baixo.</t>
+          <t>Drop set: tudo na MESMA série, reduz a carga sem descanso (15 → 12 → 10) até a falha.</t>
         </is>
       </c>
     </row>
@@ -3697,27 +3707,27 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Pullover na polia</t>
+          <t>Barra fixa ou puxada alta (pegada aberta)</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Costas</t>
+          <t>Costas · principal</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>12/10/8/8</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>Sente o dorsal alongar e contrair, cotovelos semi-fixos.</t>
+          <t>Progressão de carga ao longo das séries.</t>
         </is>
       </c>
     </row>
@@ -3739,7 +3749,7 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Remada unilateral com halter (serrote)</t>
+          <t>Remada sentada na máquina (pegada neutra)</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
@@ -3749,17 +3759,17 @@
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>10 cada</t>
+          <t>12/10/10/08</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>Um lado de cada vez, sem rodar o tronco.</t>
+          <t>Progressão de carga. Controla a fase negativa.</t>
         </is>
       </c>
     </row>
@@ -3781,12 +3791,12 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Rosca scott (banco)</t>
+          <t>Remada cavalinho (T-bar)</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Bíceps</t>
+          <t>Costas</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
@@ -3801,7 +3811,7 @@
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>Progressão de carga: aumente o peso a cada série. Cotovelos apoiados no banco, sobe e desce controlado.</t>
+          <t>Peito apoiado, puxa com os cotovelos.</t>
         </is>
       </c>
     </row>
@@ -3813,37 +3823,37 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>C · Sex · Pernas</t>
+          <t>B · Qui · Costas</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Leg press 45°</t>
+          <t>Puxada com triângulo (pegada neutra)</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Pernas · principal</t>
+          <t>Costas</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>12/10/10/08</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>Progressão de carga. Pés na largura do quadril, desce controlado.</t>
+          <t>Leva o triângulo ao peito, escápulas pra baixo.</t>
         </is>
       </c>
     </row>
@@ -3855,22 +3865,22 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>C · Sex · Pernas</t>
+          <t>B · Qui · Costas</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Agachamento hack</t>
+          <t>Pullover na polia</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Quadríceps</t>
+          <t>Costas</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
@@ -3880,12 +3890,12 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>10-12</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>Máquina, poupando a coluna que o CrossFit já castiga.</t>
+          <t>Sente o dorsal alongar e contrair, cotovelos semi-fixos.</t>
         </is>
       </c>
     </row>
@@ -3897,22 +3907,22 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>C · Sex · Pernas</t>
+          <t>B · Qui · Costas</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Cadeira extensora</t>
+          <t>Remada unilateral com halter (serrote)</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Quadríceps</t>
+          <t>Costas</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
@@ -3922,12 +3932,12 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>15/12/10</t>
+          <t>10 cada</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>Drop set: tudo na MESMA série, reduz a carga sem descanso (15 → 12 → 10) até a falha.</t>
+          <t>Um lado de cada vez, sem rodar o tronco.</t>
         </is>
       </c>
     </row>
@@ -3939,37 +3949,37 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>C · Sex · Pernas</t>
+          <t>B · Qui · Costas</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Mesa flexora (posterior)</t>
+          <t>Rosca scott (banco)</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Posterior</t>
+          <t>Bíceps</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>12/10/10/10</t>
+          <t>10-12</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>Progressão de carga. Controla a fase negativa.</t>
+          <t>Progressão de carga: aumente o peso a cada série. Cotovelos apoiados no banco, sobe e desce controlado.</t>
         </is>
       </c>
     </row>
@@ -3991,27 +4001,27 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Coice de glúteo na polia</t>
+          <t>Leg press 45°</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Glúteos</t>
+          <t>Pernas · principal</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>12 cada</t>
+          <t>12/10/10/08</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>Um lado de cada vez, segura 1 seg na contração do glúteo.</t>
+          <t>Progressão de carga. Pés na largura do quadril, desce controlado.</t>
         </is>
       </c>
     </row>
@@ -4033,12 +4043,12 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Elevação pélvica (glúteo)</t>
+          <t>Agachamento hack</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Glúteos</t>
+          <t>Quadríceps</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
@@ -4048,12 +4058,12 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10-12</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>Segura 2 seg no topo (isometria) apertando o glúteo.</t>
+          <t>Máquina, poupando a coluna que o CrossFit já castiga.</t>
         </is>
       </c>
     </row>
@@ -4075,27 +4085,27 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Panturrilha em pé</t>
+          <t>Cadeira extensora</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Panturrilha</t>
+          <t>Quadríceps</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>20/15/12/12</t>
+          <t>15/12/10</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>Drop set na última série + isometria de 2 seg no topo de cada rep.</t>
+          <t>Drop set: tudo na MESMA série, reduz a carga sem descanso (15 → 12 → 10) até a falha.</t>
         </is>
       </c>
     </row>
@@ -4107,32 +4117,37 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>D · Sáb · Corrida</t>
+          <t>C · Sex · Pernas</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Aquecimento</t>
+          <t>Mesa flexora (posterior)</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Corrida · aquecimento</t>
+          <t>Posterior</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>4</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>5 min</t>
+          <t>12/10/10/10</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>Faça o aquecimento, depois SÓ o bloco da semana atual do seu ciclo, e termine no desaquecimento. A cada 4 semanas o ciclo recomeça, subindo cerca de 10%. Comece com caminhada rápida evoluindo para trote leve.</t>
+          <t>Progressão de carga. Controla a fase negativa.</t>
         </is>
       </c>
     </row>
@@ -4144,32 +4159,37 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>D · Sáb · Corrida</t>
+          <t>C · Sex · Pernas</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Semana 1 · Corrida contínua leve</t>
+          <t>Coice de glúteo na polia</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Corrida · Semana 1</t>
+          <t>Glúteos</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>3</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>4-5 km</t>
+          <t>12 cada</t>
         </is>
       </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t>Ritmo de conversa (Z2): você consegue falar frases inteiras. Registre seu tempo total no fim.</t>
+          <t>Um lado de cada vez, segura 1 seg na contração do glúteo.</t>
         </is>
       </c>
     </row>
@@ -4181,37 +4201,37 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>D · Sáb · Corrida</t>
+          <t>C · Sex · Pernas</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Semana 2 · Fartlek</t>
+          <t>Elevação pélvica (glúteo)</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Corrida · Semana 2</t>
+          <t>Glúteos</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>(3 min corrida + 1 min caminhada)</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>6 blocos de 3 min correndo moderado + 1 min caminhando. Registre o tempo total.</t>
+          <t>Segura 2 seg no topo (isometria) apertando o glúteo.</t>
         </is>
       </c>
     </row>
@@ -4223,32 +4243,37 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>D · Sáb · Corrida</t>
+          <t>C · Sex · Pernas</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Semana 3 · Longão leve</t>
+          <t>Panturrilha em pé</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Corrida · Semana 3</t>
+          <t>Panturrilha</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>4</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>5-6 km</t>
+          <t>20/15/12/12</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>Contínuo em Z2, sem pressa, construindo resistência. Registre seu tempo.</t>
+          <t>Drop set na última série + isometria de 2 seg no topo de cada rep.</t>
         </is>
       </c>
     </row>
@@ -4270,22 +4295,22 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Semana 4 · Progressiva</t>
+          <t>Aquecimento</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Corrida · Semana 4</t>
+          <t>Corrida · aquecimento</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>5 km</t>
+          <t>5 min</t>
         </is>
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>Comece leve e termine o último km mais forte (limiar leve). Registre seu tempo.</t>
+          <t>Faça o aquecimento, depois SÓ o bloco da semana atual do seu ciclo, e termine no desaquecimento. A cada 4 semanas o ciclo recomeça, subindo cerca de 10%. Comece com caminhada rápida evoluindo para trote leve.</t>
         </is>
       </c>
     </row>
@@ -4307,180 +4332,175 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Desaquecimento</t>
+          <t>Semana 1 · Corrida contínua leve</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Corrida · volta à calma</t>
+          <t>Corrida · Semana 1</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>5 min</t>
+          <t>4-5 km</t>
         </is>
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>Trote bem leve até virar caminhada, depois alongue panturrilha, posterior e quadril.</t>
+          <t>Ritmo de conversa (Z2): você consegue falar frases inteiras. Registre seu tempo total no fim.</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Jaqueline Galo</t>
+          <t>Felipe</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>A · Quadríceps</t>
+          <t>D · Sáb · Corrida</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Agachamento cálice</t>
+          <t>Semana 2 · Fartlek</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Quadríceps</t>
+          <t>Corrida · Semana 2</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>6</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>(3 min corrida + 1 min caminhada)</t>
+        </is>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>6 blocos de 3 min correndo moderado + 1 min caminhando. Registre o tempo total.</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Jaqueline Galo</t>
+          <t>Felipe</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>A · Quadríceps</t>
+          <t>D · Sáb · Corrida</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Afundo alternado no step</t>
+          <t>Semana 3 · Longão leve</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Pernas/glúteos</t>
-        </is>
-      </c>
-      <c r="F81" t="inlineStr">
-        <is>
-          <t>3</t>
+          <t>Corrida · Semana 3</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>5-6 km</t>
+        </is>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>Contínuo em Z2, sem pressa, construindo resistência. Registre seu tempo.</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Jaqueline Galo</t>
+          <t>Felipe</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>A · Quadríceps</t>
+          <t>D · Sáb · Corrida</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Cadeira extensora</t>
+          <t>Semana 4 · Progressiva</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Quadríceps</t>
-        </is>
-      </c>
-      <c r="F82" t="inlineStr">
-        <is>
-          <t>4</t>
+          <t>Corrida · Semana 4</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>15/12/10/08</t>
+          <t>5 km</t>
         </is>
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>Progressão de carga ao longo das séries.</t>
+          <t>Comece leve e termine o último km mais forte (limiar leve). Registre seu tempo.</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Jaqueline Galo</t>
+          <t>Felipe</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>A · Quadríceps</t>
+          <t>D · Sáb · Corrida</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Leg press 45°</t>
+          <t>Desaquecimento</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Pernas</t>
-        </is>
-      </c>
-      <c r="F83" t="inlineStr">
-        <is>
-          <t>3</t>
+          <t>Corrida · volta à calma</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>5 min</t>
         </is>
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>Descida lenta (controlada).</t>
+          <t>Trote bem leve até virar caminhada, depois alongue panturrilha, posterior e quadril.</t>
         </is>
       </c>
     </row>
@@ -4502,17 +4522,22 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Escada</t>
+          <t>Agachamento cálice</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Cardio</t>
+          <t>Quadríceps</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>3</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>15 min</t>
+          <t>15</t>
         </is>
       </c>
     </row>
@@ -4524,37 +4549,32 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>B · Superiores</t>
+          <t>A · Quadríceps</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Puxador costas no graviton + Desenvolvimento halteres fechado</t>
+          <t>Afundo alternado no step</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Costas/Ombro</t>
+          <t>Pernas/glúteos</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>máximo / 10</t>
-        </is>
-      </c>
-      <c r="I85" t="inlineStr">
-        <is>
-          <t>Bi-set: sem descanso entre os dois — puxador no graviton até o máximo, seguido de desenvolvimento com halteres fechado (10 reps).</t>
+          <t>10</t>
         </is>
       </c>
     </row>
@@ -4566,37 +4586,37 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>B · Superiores</t>
+          <t>A · Quadríceps</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Pulldown barra reta (pulley) + Tríceps pulley</t>
+          <t>Cadeira extensora</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Costas/Tríceps</t>
+          <t>Quadríceps</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>15/12/10/08</t>
         </is>
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>Bi-set: sem descanso entre os dois.</t>
+          <t>Progressão de carga ao longo das séries.</t>
         </is>
       </c>
     </row>
@@ -4608,22 +4628,22 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>B · Superiores</t>
+          <t>A · Quadríceps</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Supino inclinado halteres + Rosca direta halteres</t>
+          <t>Leg press 45°</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Peito/Bíceps</t>
+          <t>Pernas</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
@@ -4638,7 +4658,7 @@
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>Bi-set: sem descanso entre os dois.</t>
+          <t>Descida lenta (controlada).</t>
         </is>
       </c>
     </row>
@@ -4650,37 +4670,27 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>B · Superiores</t>
+          <t>A · Quadríceps</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Abdominal remador</t>
+          <t>Escada</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Core</t>
-        </is>
-      </c>
-      <c r="F88" t="inlineStr">
-        <is>
-          <t>3</t>
+          <t>Cardio</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="I88" t="inlineStr">
-        <is>
-          <t>Carga: 2 kg.</t>
+          <t>15 min</t>
         </is>
       </c>
     </row>
@@ -4692,22 +4702,22 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>C · Posterior/Glúteos</t>
+          <t>B · Superiores</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Agachamento sumô halteres</t>
+          <t>Puxador costas no graviton + Desenvolvimento halteres fechado</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Pernas/glúteos</t>
+          <t>Costas/Ombro</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
@@ -4717,7 +4727,12 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>8 a 10</t>
+          <t>máximo / 10</t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>Bi-set: sem descanso entre os dois — puxador no graviton até o máximo, seguido de desenvolvimento com halteres fechado (10 reps).</t>
         </is>
       </c>
     </row>
@@ -4729,22 +4744,22 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>C · Posterior/Glúteos</t>
+          <t>B · Superiores</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Cadeira flexora</t>
+          <t>Pulldown barra reta (pulley) + Tríceps pulley</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Posterior de coxa</t>
+          <t>Costas/Tríceps</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
@@ -4754,12 +4769,12 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>15/12/10</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I90" t="inlineStr">
         <is>
-          <t>Progressão de carga ao longo das séries.</t>
+          <t>Bi-set: sem descanso entre os dois.</t>
         </is>
       </c>
     </row>
@@ -4771,22 +4786,22 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>C · Posterior/Glúteos</t>
+          <t>B · Superiores</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Glúteo chute no pulley</t>
+          <t>Supino inclinado halteres + Rosca direta halteres</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>Glúteos</t>
+          <t>Peito/Bíceps</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
@@ -4797,6 +4812,11 @@
       <c r="G91" t="inlineStr">
         <is>
           <t>15</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>Bi-set: sem descanso entre os dois.</t>
         </is>
       </c>
     </row>
@@ -4808,22 +4828,22 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>C · Posterior/Glúteos</t>
+          <t>B · Superiores</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Cadeira abdutora</t>
+          <t>Abdominal remador</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Glúteos · abdutores</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
@@ -4834,6 +4854,11 @@
       <c r="G92" t="inlineStr">
         <is>
           <t>15</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>Carga: 2 kg.</t>
         </is>
       </c>
     </row>
@@ -4855,17 +4880,22 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Escada intervalada</t>
+          <t>Agachamento sumô halteres</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Cardio</t>
+          <t>Pernas/glúteos</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>4</t>
         </is>
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>2 min leve / 2 min forte × 6</t>
+          <t>8 a 10</t>
         </is>
       </c>
     </row>
@@ -4877,22 +4907,22 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>D · Circuito Full Body</t>
+          <t>C · Posterior/Glúteos</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Flexão de braço de joelhos</t>
+          <t>Cadeira flexora</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>Peito/Core</t>
+          <t>Posterior de coxa</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
@@ -4902,12 +4932,12 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>15/12/10</t>
         </is>
       </c>
       <c r="I94" t="inlineStr">
         <is>
-          <t>Circuito: repetir os 5 exercícios em sequência, 3 voltas — 30s de descanso entre exercícios e 2 min entre as voltas. Sem carga (peso do corpo).</t>
+          <t>Progressão de carga ao longo das séries.</t>
         </is>
       </c>
     </row>
@@ -4919,22 +4949,22 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>D · Circuito Full Body</t>
+          <t>C · Posterior/Glúteos</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Step-up no box</t>
+          <t>Glúteo chute no pulley</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>Pernas/glúteos</t>
+          <t>Glúteos</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
@@ -4944,7 +4974,7 @@
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>10 cada perna</t>
+          <t>15</t>
         </is>
       </c>
     </row>
@@ -4956,22 +4986,22 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>D · Circuito Full Body</t>
+          <t>C · Posterior/Glúteos</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Senta e levanta com halteres no box</t>
+          <t>Cadeira abdutora</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>Pernas/glúteos</t>
+          <t>Glúteos · abdutores</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
@@ -4993,17 +5023,17 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>D · Circuito Full Body</t>
+          <t>C · Posterior/Glúteos</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Mountain climber no box</t>
+          <t>Escada intervalada</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
@@ -5011,14 +5041,9 @@
           <t>Cardio</t>
         </is>
       </c>
-      <c r="F97" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>40s</t>
+          <t>2 min leve / 2 min forte × 6</t>
         </is>
       </c>
     </row>
@@ -5040,12 +5065,12 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Abdominal curto no solo</t>
+          <t>Flexão de braço de joelhos</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>Core</t>
+          <t>Peito/Core</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
@@ -5055,145 +5080,145 @@
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>Circuito: repetir os 5 exercícios em sequência, 3 voltas — 30s de descanso entre exercícios e 2 min entre as voltas. Sem carga (peso do corpo).</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Lara</t>
+          <t>Jaqueline Galo</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>A · Tiros longos na esteira + core</t>
+          <t>D · Circuito Full Body</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Esteira — aquecimento progressivo</t>
+          <t>Step-up no box</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Cardio · aquecimento</t>
+          <t>Pernas/glúteos</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>3</t>
         </is>
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>10 min</t>
-        </is>
-      </c>
-      <c r="I99" t="inlineStr">
-        <is>
-          <t>Comece em caminhada e aumente o ritmo aos poucos até um trote confortável, preparando o corpo para os tiros.</t>
+          <t>10 cada perna</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Lara</t>
+          <t>Jaqueline Galo</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>A · Tiros longos na esteira + core</t>
+          <t>D · Circuito Full Body</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Esteira — tiros de 800m</t>
+          <t>Senta e levanta com halteres no box</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>Cardio · intervalado</t>
+          <t>Pernas/glúteos</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>800m forte</t>
-        </is>
-      </c>
-      <c r="I100" t="inlineStr">
-        <is>
-          <t>Cada tiro de 800m em ritmo forte, bem acima do confortável. Recuperação de 2–3 min em caminhada entre os tiros. Repita 4x.</t>
+          <t>15</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Lara</t>
+          <t>Jaqueline Galo</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>A · Tiros longos na esteira + core</t>
+          <t>D · Circuito Full Body</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Esteira — desaquecimento</t>
+          <t>Mountain climber no box</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>Cardio · desaquecimento</t>
+          <t>Cardio</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>3</t>
         </is>
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>5 min</t>
-        </is>
-      </c>
-      <c r="I101" t="inlineStr">
-        <is>
-          <t>Trote leve reduzindo o ritmo aos poucos. Finalize com alongamento de pernas.</t>
+          <t>40s</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Lara</t>
+          <t>Jaqueline Galo</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>A · Tiros longos na esteira + core</t>
+          <t>D · Circuito Full Body</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>Prancha abdominal</t>
+          <t>Abdominal curto no solo</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
@@ -5203,17 +5228,12 @@
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>1 min</t>
-        </is>
-      </c>
-      <c r="I102" t="inlineStr">
-        <is>
-          <t>Corpo alinhado da cabeça ao calcanhar, abdômen contraído.</t>
+          <t>20</t>
         </is>
       </c>
     </row>
@@ -5235,27 +5255,22 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>Abdominal oblíquo (bicicleta)</t>
+          <t>Esteira — aquecimento progressivo</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Core · oblíquos</t>
-        </is>
-      </c>
-      <c r="F103" t="inlineStr">
-        <is>
-          <t>4</t>
+          <t>Cardio · aquecimento</t>
         </is>
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>10 min</t>
         </is>
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>Alterne cotovelo–joelho oposto, movimento controlado, sem puxar o pescoço.</t>
+          <t>Comece em caminhada e aumente o ritmo aos poucos até um trote confortável, preparando o corpo para os tiros.</t>
         </is>
       </c>
     </row>
@@ -5267,22 +5282,22 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>B · Inferiores</t>
+          <t>A · Tiros longos na esteira + core</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>Leg press horizontal</t>
+          <t>Esteira — tiros de 800m</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Pernas · principal</t>
+          <t>Cardio · intervalado</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
@@ -5292,12 +5307,12 @@
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>15/12/10/08</t>
+          <t>800m forte</t>
         </is>
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>Progressão de carga ao longo das séries (pirâmide): aumenta a carga e diminui as reps a cada série.</t>
+          <t>Cada tiro de 800m em ritmo forte, bem acima do confortável. Recuperação de 2–3 min em caminhada entre os tiros. Repita 4x.</t>
         </is>
       </c>
     </row>
@@ -5309,37 +5324,32 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>B · Inferiores</t>
+          <t>A · Tiros longos na esteira + core</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Cadeira extensora</t>
+          <t>Esteira — desaquecimento</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>Quadríceps</t>
-        </is>
-      </c>
-      <c r="F105" t="inlineStr">
-        <is>
-          <t>4</t>
+          <t>Cardio · desaquecimento</t>
         </is>
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>5 min</t>
         </is>
       </c>
       <c r="I105" t="inlineStr">
         <is>
-          <t>Movimento controlado, sem dar impulso; segure meio segundo no topo.</t>
+          <t>Trote leve reduzindo o ritmo aos poucos. Finalize com alongamento de pernas.</t>
         </is>
       </c>
     </row>
@@ -5351,22 +5361,22 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>B · Inferiores</t>
+          <t>A · Tiros longos na esteira + core</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>Cadeira flexora</t>
+          <t>Prancha abdominal</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>Posterior de coxa</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="F106" t="inlineStr">
@@ -5376,12 +5386,12 @@
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>1 min</t>
         </is>
       </c>
       <c r="I106" t="inlineStr">
         <is>
-          <t>Movimento controlado, segurar 1s na contração.</t>
+          <t>Corpo alinhado da cabeça ao calcanhar, abdômen contraído.</t>
         </is>
       </c>
     </row>
@@ -5393,22 +5403,22 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>B · Inferiores</t>
+          <t>A · Tiros longos na esteira + core</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>Panturrilha em pé na máquina</t>
+          <t>Abdominal oblíquo (bicicleta)</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>Panturrilha · tríceps sural</t>
+          <t>Core · oblíquos</t>
         </is>
       </c>
       <c r="F107" t="inlineStr">
@@ -5423,7 +5433,7 @@
       </c>
       <c r="I107" t="inlineStr">
         <is>
-          <t>Amplitude total, subir bem no topo e segurar 1s.</t>
+          <t>Alterne cotovelo–joelho oposto, movimento controlado, sem puxar o pescoço.</t>
         </is>
       </c>
     </row>
@@ -5445,27 +5455,27 @@
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>Bike — HIIT</t>
+          <t>Leg press horizontal</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>Cardio · intervalado</t>
+          <t>Pernas · principal</t>
         </is>
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t>3 min pesado + 2 min devagar</t>
+          <t>15/12/10/08</t>
         </is>
       </c>
       <c r="I108" t="inlineStr">
         <is>
-          <t>6 tiros: 3 min em ritmo pesado + 2 min devagar sem carga (recuperação ativa). Repita os 6 blocos (~30 min no total).</t>
+          <t>Progressão de carga ao longo das séries (pirâmide): aumenta a carga e diminui as reps a cada série.</t>
         </is>
       </c>
     </row>
@@ -5477,22 +5487,22 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>C · Circuito de braço + tiros</t>
+          <t>B · Inferiores</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>Puxador frente delta + Rosca direta (bi-set)</t>
+          <t>Cadeira extensora</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>Dorsais · bíceps</t>
+          <t>Quadríceps</t>
         </is>
       </c>
       <c r="F109" t="inlineStr">
@@ -5502,12 +5512,12 @@
       </c>
       <c r="G109" t="inlineStr">
         <is>
-          <t>15 / 20</t>
+          <t>20</t>
         </is>
       </c>
       <c r="I109" t="inlineStr">
         <is>
-          <t>Bi-set sem descanso: puxador frente com pegada delta 15 reps, emenda rosca direta com halteres 20 reps. Descanse e repita 4x.</t>
+          <t>Movimento controlado, sem dar impulso; segure meio segundo no topo.</t>
         </is>
       </c>
     </row>
@@ -5519,37 +5529,37 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>C · Circuito de braço + tiros</t>
+          <t>B · Inferiores</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>Esteira — 800m</t>
+          <t>Cadeira flexora</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>Cardio · intervalado</t>
+          <t>Posterior de coxa</t>
         </is>
       </c>
       <c r="F110" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G110" t="inlineStr">
         <is>
-          <t>800m forte</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I110" t="inlineStr">
         <is>
-          <t>Tiro de 800m em ritmo forte logo depois do bi-set.</t>
+          <t>Movimento controlado, segurar 1s na contração.</t>
         </is>
       </c>
     </row>
@@ -5561,22 +5571,22 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>C · Circuito de braço + tiros</t>
+          <t>B · Inferiores</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>Remada sentada + Desenvolvimento com halteres em pé (bi-set)</t>
+          <t>Panturrilha em pé na máquina</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>Costas · ombro</t>
+          <t>Panturrilha · tríceps sural</t>
         </is>
       </c>
       <c r="F111" t="inlineStr">
@@ -5586,12 +5596,12 @@
       </c>
       <c r="G111" t="inlineStr">
         <is>
-          <t>15 cada</t>
+          <t>20</t>
         </is>
       </c>
       <c r="I111" t="inlineStr">
         <is>
-          <t>Bi-set sem descanso: remada sentada 15 reps, emenda desenvolvimento com halteres em pé 15 reps. Repita 4x.</t>
+          <t>Amplitude total, subir bem no topo e segurar 1s.</t>
         </is>
       </c>
     </row>
@@ -5603,17 +5613,17 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>C · Circuito de braço + tiros</t>
+          <t>B · Inferiores</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>Esteira — 800m</t>
+          <t>Bike — HIIT</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
@@ -5623,17 +5633,17 @@
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>6</t>
         </is>
       </c>
       <c r="G112" t="inlineStr">
         <is>
-          <t>800m forte</t>
+          <t>3 min pesado + 2 min devagar</t>
         </is>
       </c>
       <c r="I112" t="inlineStr">
         <is>
-          <t>Tiro de 800m em ritmo forte.</t>
+          <t>6 tiros: 3 min em ritmo pesado + 2 min devagar sem carga (recuperação ativa). Repita os 6 blocos (~30 min no total).</t>
         </is>
       </c>
     </row>
@@ -5655,12 +5665,12 @@
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>Supino sentado na máquina + Tríceps francês com halteres (bi-set)</t>
+          <t>Puxador frente delta + Rosca direta (bi-set)</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>Peitoral · tríceps</t>
+          <t>Dorsais · bíceps</t>
         </is>
       </c>
       <c r="F113" t="inlineStr">
@@ -5670,12 +5680,12 @@
       </c>
       <c r="G113" t="inlineStr">
         <is>
-          <t>15 cada</t>
+          <t>15 / 20</t>
         </is>
       </c>
       <c r="I113" t="inlineStr">
         <is>
-          <t>Bi-set sem descanso: supino sentado na máquina 15 reps, emenda tríceps francês com halteres 15 reps. Repita 4x.</t>
+          <t>Bi-set sem descanso: puxador frente com pegada delta 15 reps, emenda rosca direta com halteres 20 reps. Descanse e repita 4x.</t>
         </is>
       </c>
     </row>
@@ -5717,7 +5727,7 @@
       </c>
       <c r="I114" t="inlineStr">
         <is>
-          <t>Último tiro de 800m em ritmo forte.</t>
+          <t>Tiro de 800m em ritmo forte logo depois do bi-set.</t>
         </is>
       </c>
     </row>
@@ -5739,12 +5749,12 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>Abdominal curto com peso</t>
+          <t>Remada sentada + Desenvolvimento com halteres em pé (bi-set)</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>Core</t>
+          <t>Costas · ombro</t>
         </is>
       </c>
       <c r="F115" t="inlineStr">
@@ -5754,12 +5764,12 @@
       </c>
       <c r="G115" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>15 cada</t>
         </is>
       </c>
       <c r="I115" t="inlineStr">
         <is>
-          <t>Segure o peso no peito, contraia o abdômen no topo sem puxar o pescoço.</t>
+          <t>Bi-set sem descanso: remada sentada 15 reps, emenda desenvolvimento com halteres em pé 15 reps. Repita 4x.</t>
         </is>
       </c>
     </row>
@@ -5771,32 +5781,37 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>D · Corrida + glúteos</t>
+          <t>C · Circuito de braço + tiros</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>Esteira — corrida contínua</t>
+          <t>Esteira — 800m</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>Cardio · aeróbico</t>
+          <t>Cardio · intervalado</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>1</t>
         </is>
       </c>
       <c r="G116" t="inlineStr">
         <is>
-          <t>3 km sem parar</t>
+          <t>800m forte</t>
         </is>
       </c>
       <c r="I116" t="inlineStr">
         <is>
-          <t>Ritmo moderado e constante, sem pausa. Respiração controlada — dá pra manter conversa curta.</t>
+          <t>Tiro de 800m em ritmo forte.</t>
         </is>
       </c>
     </row>
@@ -5808,22 +5823,22 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>D · Corrida + glúteos</t>
+          <t>C · Circuito de braço + tiros</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>Agachamento sumô com kettlebell</t>
+          <t>Supino sentado na máquina + Tríceps francês com halteres (bi-set)</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>Glúteos/pernas · principal</t>
+          <t>Peitoral · tríceps</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
@@ -5833,12 +5848,12 @@
       </c>
       <c r="G117" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>15 cada</t>
         </is>
       </c>
       <c r="I117" t="inlineStr">
         <is>
-          <t>Pés afastados e pontas abertas; desça mantendo o tronco ereto e o peso no calcanhar.</t>
+          <t>Bi-set sem descanso: supino sentado na máquina 15 reps, emenda tríceps francês com halteres 15 reps. Repita 4x.</t>
         </is>
       </c>
     </row>
@@ -5850,37 +5865,37 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>D · Corrida + glúteos</t>
+          <t>C · Circuito de braço + tiros</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>Cadeira abdutora</t>
+          <t>Esteira — 800m</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>Glúteos · abdutores</t>
+          <t>Cardio · intervalado</t>
         </is>
       </c>
       <c r="F118" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G118" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>800m forte</t>
         </is>
       </c>
       <c r="I118" t="inlineStr">
         <is>
-          <t>Abrir as pernas com controle, sem jogar o tronco para trás.</t>
+          <t>Último tiro de 800m em ritmo forte.</t>
         </is>
       </c>
     </row>
@@ -5892,22 +5907,22 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>D · Corrida + glúteos</t>
+          <t>C · Circuito de braço + tiros</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>Glúteo coice na polia</t>
+          <t>Abdominal curto com peso</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>Glúteos</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="F119" t="inlineStr">
@@ -5922,7 +5937,7 @@
       </c>
       <c r="I119" t="inlineStr">
         <is>
-          <t>Movimento controlado; contraia o glúteo no topo sem hiperestender a lombar.</t>
+          <t>Segure o peso no peito, contraia o abdômen no topo sem puxar o pescoço.</t>
         </is>
       </c>
     </row>
@@ -5944,96 +5959,91 @@
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>Prancha abdominal</t>
+          <t>Esteira — corrida contínua</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>Core</t>
-        </is>
-      </c>
-      <c r="F120" t="inlineStr">
-        <is>
-          <t>4</t>
+          <t>Cardio · aeróbico</t>
         </is>
       </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t>1 min</t>
+          <t>3 km sem parar</t>
         </is>
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>Corpo alinhado da cabeça ao calcanhar, abdômen contraído.</t>
+          <t>Ritmo moderado e constante, sem pausa. Respiração controlada — dá pra manter conversa curta.</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>Marina Barbato</t>
+          <t>Lara</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>A · Seg · Quadríceps</t>
+          <t>D · Corrida + glúteos</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>Agachamento livre (ativação)</t>
+          <t>Agachamento sumô com kettlebell</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>Quadríceps</t>
+          <t>Glúteos/pernas · principal</t>
         </is>
       </c>
       <c r="F121" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G121" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I121" t="inlineStr">
         <is>
-          <t>Descida lenta (excêntrica controlada) — séries de ativação antes da carga.</t>
+          <t>Pés afastados e pontas abertas; desça mantendo o tronco ereto e o peso no calcanhar.</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>Marina Barbato</t>
+          <t>Lara</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>A · Seg · Quadríceps</t>
+          <t>D · Corrida + glúteos</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>Agachamento livre (carga)</t>
+          <t>Cadeira abdutora</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>Quadríceps</t>
+          <t>Glúteos · abdutores</t>
         </is>
       </c>
       <c r="F122" t="inlineStr">
@@ -6043,81 +6053,81 @@
       </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I122" t="inlineStr">
         <is>
-          <t>Séries de trabalho, na sequência das 2 séries de ativação.</t>
+          <t>Abrir as pernas com controle, sem jogar o tronco para trás.</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>Marina Barbato</t>
+          <t>Lara</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>A · Seg · Quadríceps</t>
+          <t>D · Corrida + glúteos</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>Leg press 45°</t>
+          <t>Glúteo coice na polia</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>Quadríceps</t>
+          <t>Glúteos</t>
         </is>
       </c>
       <c r="F123" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G123" t="inlineStr">
         <is>
-          <t>20/15/12/10/8</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I123" t="inlineStr">
         <is>
-          <t>Progressão de carga a cada série.</t>
+          <t>Movimento controlado; contraia o glúteo no topo sem hiperestender a lombar.</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>Marina Barbato</t>
+          <t>Lara</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>A · Seg · Quadríceps</t>
+          <t>D · Corrida + glúteos</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>Cadeira extensora</t>
+          <t>Prancha abdominal</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>Quadríceps</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="F124" t="inlineStr">
@@ -6127,7 +6137,12 @@
       </c>
       <c r="G124" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>1 min</t>
+        </is>
+      </c>
+      <c r="I124" t="inlineStr">
+        <is>
+          <t>Corpo alinhado da cabeça ao calcanhar, abdômen contraído.</t>
         </is>
       </c>
     </row>
@@ -6149,7 +6164,7 @@
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>Cadeira extensora</t>
+          <t>Agachamento livre (ativação)</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
@@ -6159,17 +6174,17 @@
       </c>
       <c r="F125" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G125" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>20</t>
         </is>
       </c>
       <c r="I125" t="inlineStr">
         <is>
-          <t>Segundo bloco — aumentar a carga.</t>
+          <t>Descida lenta (excêntrica controlada) — séries de ativação antes da carga.</t>
         </is>
       </c>
     </row>
@@ -6191,12 +6206,12 @@
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>Panturrilha em pé</t>
+          <t>Agachamento livre (carga)</t>
         </is>
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>Panturrilha</t>
+          <t>Quadríceps</t>
         </is>
       </c>
       <c r="F126" t="inlineStr">
@@ -6206,7 +6221,12 @@
       </c>
       <c r="G126" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>Séries de trabalho, na sequência das 2 séries de ativação.</t>
         </is>
       </c>
     </row>
@@ -6218,37 +6238,37 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>B · Ter · Dorsal</t>
+          <t>A · Seg · Quadríceps</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>Remada sentada pulley</t>
+          <t>Leg press 45°</t>
         </is>
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>Dorsal</t>
+          <t>Quadríceps</t>
         </is>
       </c>
       <c r="F127" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="G127" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>20/15/12/10/8</t>
         </is>
       </c>
       <c r="I127" t="inlineStr">
         <is>
-          <t>Bi-set com a rosca direta com halteres (próximo exercício), sem descanso entre eles.</t>
+          <t>Progressão de carga a cada série.</t>
         </is>
       </c>
     </row>
@@ -6260,22 +6280,22 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>B · Ter · Dorsal</t>
+          <t>A · Seg · Quadríceps</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>Rosca direta halteres</t>
+          <t>Cadeira extensora</t>
         </is>
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>Bíceps</t>
+          <t>Quadríceps</t>
         </is>
       </c>
       <c r="F128" t="inlineStr">
@@ -6286,11 +6306,6 @@
       <c r="G128" t="inlineStr">
         <is>
           <t>20</t>
-        </is>
-      </c>
-      <c r="I128" t="inlineStr">
-        <is>
-          <t>Bi-set com a remada sentada pulley (exercício anterior).</t>
         </is>
       </c>
     </row>
@@ -6302,22 +6317,22 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>B · Ter · Dorsal</t>
+          <t>A · Seg · Quadríceps</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>Puxador aberto pulley</t>
+          <t>Cadeira extensora</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>Dorsal</t>
+          <t>Quadríceps</t>
         </is>
       </c>
       <c r="F129" t="inlineStr">
@@ -6327,12 +6342,12 @@
       </c>
       <c r="G129" t="inlineStr">
         <is>
-          <t>15/12/10/8</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I129" t="inlineStr">
         <is>
-          <t>Progressão de carga a cada série.</t>
+          <t>Segundo bloco — aumentar a carga.</t>
         </is>
       </c>
     </row>
@@ -6344,32 +6359,32 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>B · Ter · Dorsal</t>
+          <t>A · Seg · Quadríceps</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>Remo aeróbico</t>
+          <t>Panturrilha em pé</t>
         </is>
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>Cardio</t>
+          <t>Panturrilha</t>
+        </is>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>4</t>
         </is>
       </c>
       <c r="G130" t="inlineStr">
         <is>
-          <t>10 min</t>
-        </is>
-      </c>
-      <c r="I130" t="inlineStr">
-        <is>
-          <t>Ritmo moderado-intenso.</t>
+          <t>20</t>
         </is>
       </c>
     </row>
@@ -6391,12 +6406,12 @@
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>Banco romano</t>
+          <t>Remada sentada pulley</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>Lombar/Posterior</t>
+          <t>Dorsal</t>
         </is>
       </c>
       <c r="F131" t="inlineStr">
@@ -6406,12 +6421,12 @@
       </c>
       <c r="G131" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>20</t>
         </is>
       </c>
       <c r="I131" t="inlineStr">
         <is>
-          <t>Descida lenta (excêntrica controlada).</t>
+          <t>Bi-set com a rosca direta com halteres (próximo exercício), sem descanso entre eles.</t>
         </is>
       </c>
     </row>
@@ -6423,22 +6438,22 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>C · Qua · Posterior de coxa</t>
+          <t>B · Ter · Dorsal</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>Mesa flexora</t>
+          <t>Rosca direta halteres</t>
         </is>
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>Posterior de coxa</t>
+          <t>Bíceps</t>
         </is>
       </c>
       <c r="F132" t="inlineStr">
@@ -6449,6 +6464,11 @@
       <c r="G132" t="inlineStr">
         <is>
           <t>20</t>
+        </is>
+      </c>
+      <c r="I132" t="inlineStr">
+        <is>
+          <t>Bi-set com a remada sentada pulley (exercício anterior).</t>
         </is>
       </c>
     </row>
@@ -6460,22 +6480,22 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>C · Qua · Posterior de coxa</t>
+          <t>B · Ter · Dorsal</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>Mesa flexora</t>
+          <t>Puxador aberto pulley</t>
         </is>
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>Posterior de coxa</t>
+          <t>Dorsal</t>
         </is>
       </c>
       <c r="F133" t="inlineStr">
@@ -6485,12 +6505,12 @@
       </c>
       <c r="G133" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>15/12/10/8</t>
         </is>
       </c>
       <c r="I133" t="inlineStr">
         <is>
-          <t>Segundo bloco — aumentar a carga.</t>
+          <t>Progressão de carga a cada série.</t>
         </is>
       </c>
     </row>
@@ -6502,32 +6522,32 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>C · Qua · Posterior de coxa</t>
+          <t>B · Ter · Dorsal</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>Flexor de joelhos em pé</t>
+          <t>Remo aeróbico</t>
         </is>
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>Posterior de coxa</t>
-        </is>
-      </c>
-      <c r="F134" t="inlineStr">
-        <is>
-          <t>4</t>
+          <t>Cardio</t>
         </is>
       </c>
       <c r="G134" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>10 min</t>
+        </is>
+      </c>
+      <c r="I134" t="inlineStr">
+        <is>
+          <t>Ritmo moderado-intenso.</t>
         </is>
       </c>
     </row>
@@ -6539,22 +6559,22 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>C · Qua · Posterior de coxa</t>
+          <t>B · Ter · Dorsal</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>Stiff halteres</t>
+          <t>Banco romano</t>
         </is>
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>Posterior de coxa/Glúteo</t>
+          <t>Lombar/Posterior</t>
         </is>
       </c>
       <c r="F135" t="inlineStr">
@@ -6565,6 +6585,11 @@
       <c r="G135" t="inlineStr">
         <is>
           <t>15</t>
+        </is>
+      </c>
+      <c r="I135" t="inlineStr">
+        <is>
+          <t>Descida lenta (excêntrica controlada).</t>
         </is>
       </c>
     </row>
@@ -6586,12 +6611,12 @@
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>Abdominal máquina</t>
+          <t>Mesa flexora</t>
         </is>
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>Abdômen</t>
+          <t>Posterior de coxa</t>
         </is>
       </c>
       <c r="F136" t="inlineStr">
@@ -6601,7 +6626,7 @@
       </c>
       <c r="G136" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>20</t>
         </is>
       </c>
     </row>
@@ -6613,22 +6638,22 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>D · Qui · Ombro, Tríceps e Bíceps</t>
+          <t>C · Qua · Posterior de coxa</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>Manguito rotador (elástico ou pulley)</t>
+          <t>Mesa flexora</t>
         </is>
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>Ombro</t>
+          <t>Posterior de coxa</t>
         </is>
       </c>
       <c r="F137" t="inlineStr">
@@ -6643,7 +6668,7 @@
       </c>
       <c r="I137" t="inlineStr">
         <is>
-          <t>Ativação do manguito rotador antes da carga.</t>
+          <t>Segundo bloco — aumentar a carga.</t>
         </is>
       </c>
     </row>
@@ -6655,22 +6680,22 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>D · Qui · Ombro, Tríceps e Bíceps</t>
+          <t>C · Qua · Posterior de coxa</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>Elevação lateral halteres</t>
+          <t>Flexor de joelhos em pé</t>
         </is>
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>Ombro</t>
+          <t>Posterior de coxa</t>
         </is>
       </c>
       <c r="F138" t="inlineStr">
@@ -6680,7 +6705,7 @@
       </c>
       <c r="G138" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>15</t>
         </is>
       </c>
     </row>
@@ -6692,22 +6717,22 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>D · Qui · Ombro, Tríceps e Bíceps</t>
+          <t>C · Qua · Posterior de coxa</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>Elevação lateral no pulley</t>
+          <t>Stiff halteres</t>
         </is>
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>Ombro</t>
+          <t>Posterior de coxa/Glúteo</t>
         </is>
       </c>
       <c r="F139" t="inlineStr">
@@ -6717,7 +6742,7 @@
       </c>
       <c r="G139" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>15</t>
         </is>
       </c>
     </row>
@@ -6729,22 +6754,22 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>D · Qui · Ombro, Tríceps e Bíceps</t>
+          <t>C · Qua · Posterior de coxa</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>Desenvolvimento fechado halteres</t>
+          <t>Abdominal máquina</t>
         </is>
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>Ombro</t>
+          <t>Abdômen</t>
         </is>
       </c>
       <c r="F140" t="inlineStr">
@@ -6776,22 +6801,27 @@
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>Tríceps pulley corda</t>
+          <t>Manguito rotador (elástico ou pulley)</t>
         </is>
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>Tríceps</t>
+          <t>Ombro</t>
         </is>
       </c>
       <c r="F141" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G141" t="inlineStr">
         <is>
           <t>12</t>
+        </is>
+      </c>
+      <c r="I141" t="inlineStr">
+        <is>
+          <t>Ativação do manguito rotador antes da carga.</t>
         </is>
       </c>
     </row>
@@ -6803,22 +6833,22 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>E · Sex · Glúteos</t>
+          <t>D · Qui · Ombro, Tríceps e Bíceps</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>Supino sentada</t>
+          <t>Elevação lateral halteres</t>
         </is>
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t>Glúteo</t>
+          <t>Ombro</t>
         </is>
       </c>
       <c r="F142" t="inlineStr">
@@ -6829,11 +6859,6 @@
       <c r="G142" t="inlineStr">
         <is>
           <t>20</t>
-        </is>
-      </c>
-      <c r="I142" t="inlineStr">
-        <is>
-          <t>Confirmar nome do aparelho com a Larissa.</t>
         </is>
       </c>
     </row>
@@ -6845,22 +6870,22 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>E · Sex · Glúteos</t>
+          <t>D · Qui · Ombro, Tríceps e Bíceps</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>Cadeira abdutora</t>
+          <t>Elevação lateral no pulley</t>
         </is>
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>Glúteo médio</t>
+          <t>Ombro</t>
         </is>
       </c>
       <c r="F143" t="inlineStr">
@@ -6870,7 +6895,7 @@
       </c>
       <c r="G143" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>10</t>
         </is>
       </c>
     </row>
@@ -6882,22 +6907,22 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>E · Sex · Glúteos</t>
+          <t>D · Qui · Ombro, Tríceps e Bíceps</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>Elevação pélvica</t>
+          <t>Desenvolvimento fechado halteres</t>
         </is>
       </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t>Glúteo</t>
+          <t>Ombro</t>
         </is>
       </c>
       <c r="F144" t="inlineStr">
@@ -6907,7 +6932,7 @@
       </c>
       <c r="G144" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>15</t>
         </is>
       </c>
     </row>
@@ -6919,32 +6944,32 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>E · Sex · Glúteos</t>
+          <t>D · Qui · Ombro, Tríceps e Bíceps</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>Glúteo no pulley (extensão de quadril)</t>
+          <t>Tríceps pulley corda</t>
         </is>
       </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t>Glúteo</t>
+          <t>Tríceps</t>
         </is>
       </c>
       <c r="F145" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="G145" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>12</t>
         </is>
       </c>
     </row>
@@ -6966,20 +6991,173 @@
       </c>
       <c r="D146" t="inlineStr">
         <is>
+          <t>Supino sentada</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>Glúteo</t>
+        </is>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="I146" t="inlineStr">
+        <is>
+          <t>Confirmar nome do aparelho com a Larissa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>Marina Barbato</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>E · Sex · Glúteos</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>Cadeira abdutora</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>Glúteo médio</t>
+        </is>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>Marina Barbato</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>E · Sex · Glúteos</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>Elevação pélvica</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>Glúteo</t>
+        </is>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G148" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>Marina Barbato</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>E · Sex · Glúteos</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>Glúteo no pulley (extensão de quadril)</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>Glúteo</t>
+        </is>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>Marina Barbato</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>E · Sex · Glúteos</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
           <t>Glúteo — chute na máquina</t>
         </is>
       </c>
-      <c r="E146" t="inlineStr">
+      <c r="E150" t="inlineStr">
         <is>
           <t>Glúteo</t>
         </is>
       </c>
-      <c r="F146" t="inlineStr">
+      <c r="F150" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="G146" t="inlineStr">
+      <c r="G150" t="inlineStr">
         <is>
           <t>15</t>
         </is>

</xml_diff>